<commit_message>
TECH.OL PP&E, CHE, STD + Excel
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/TECH.OL.xlsx
+++ b/data/obx_xlsx/TECH.OL.xlsx
@@ -1401,7 +1401,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="[&gt;=100]#,###0.0\%;[&lt;=-100]-#,###0.0\%;#,###0.0\%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color rgb="FF000000"/>
@@ -1446,6 +1446,11 @@
       <sz val="10.0"/>
       <color rgb="FFF5475B"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11.0"/>
@@ -1515,7 +1520,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1597,10 +1602,11 @@
     <xf borderId="3" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
     <xf borderId="3" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="3" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -11185,9 +11191,13 @@
       <c r="B60" s="16">
         <v>170.7</v>
       </c>
-      <c r="C60" s="14"/>
-      <c r="D60" s="15">
-        <v>7.27</v>
+      <c r="C60" s="14">
+        <f t="shared" ref="C60:D60" si="1">C61+C65</f>
+        <v>174.57</v>
+      </c>
+      <c r="D60" s="27">
+        <f t="shared" si="1"/>
+        <v>166.77</v>
       </c>
       <c r="E60" s="16">
         <v>168.33</v>
@@ -11226,28 +11236,31 @@
         <v>0.22</v>
       </c>
       <c r="Q60" s="14">
-        <f t="shared" ref="Q60:R60" si="1">SUM(Q68,Q74:Q75)</f>
+        <f t="shared" ref="Q60:R60" si="2">SUM(Q68,Q74:Q75)</f>
         <v>0.5</v>
       </c>
       <c r="R60" s="15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.65</v>
       </c>
-      <c r="S60" s="15"/>
+      <c r="S60" s="15">
+        <f>(R60+T60)/2</f>
+        <v>1.88</v>
+      </c>
       <c r="T60" s="15">
-        <f t="shared" ref="T60:W60" si="2">SUM(T68,T74:T75)</f>
+        <f t="shared" ref="T60:W60" si="3">SUM(T68,T74:T75)</f>
         <v>2.11</v>
       </c>
       <c r="U60" s="15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.48</v>
       </c>
       <c r="V60" s="15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.2</v>
       </c>
       <c r="W60" s="15">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.92</v>
       </c>
     </row>
@@ -11381,7 +11394,9 @@
       <c r="C65" s="15">
         <v>7.16</v>
       </c>
-      <c r="D65" s="14"/>
+      <c r="D65" s="15">
+        <v>7.27</v>
+      </c>
       <c r="E65" s="14"/>
       <c r="F65" s="14"/>
       <c r="G65" s="14"/>
@@ -21420,2308 +21435,2308 @@
       </c>
     </row>
     <row r="19" ht="15.0" customHeight="1">
-      <c r="A19" s="27" t="s">
+      <c r="A19" s="28" t="s">
         <v>413</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
-      <c r="K19" s="28"/>
-      <c r="L19" s="28"/>
-      <c r="M19" s="28"/>
-      <c r="N19" s="28"/>
-      <c r="O19" s="28"/>
-      <c r="P19" s="28"/>
-      <c r="Q19" s="28"/>
-      <c r="R19" s="28"/>
-      <c r="S19" s="28"/>
-      <c r="T19" s="28"/>
-      <c r="U19" s="28"/>
-      <c r="V19" s="28"/>
-      <c r="W19" s="28"/>
-      <c r="X19" s="28"/>
-      <c r="Y19" s="28"/>
-      <c r="Z19" s="28"/>
-      <c r="AA19" s="28"/>
-      <c r="AB19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="29"/>
+      <c r="J19" s="29"/>
+      <c r="K19" s="29"/>
+      <c r="L19" s="29"/>
+      <c r="M19" s="29"/>
+      <c r="N19" s="29"/>
+      <c r="O19" s="29"/>
+      <c r="P19" s="29"/>
+      <c r="Q19" s="29"/>
+      <c r="R19" s="29"/>
+      <c r="S19" s="29"/>
+      <c r="T19" s="29"/>
+      <c r="U19" s="29"/>
+      <c r="V19" s="29"/>
+      <c r="W19" s="29"/>
+      <c r="X19" s="29"/>
+      <c r="Y19" s="29"/>
+      <c r="Z19" s="29"/>
+      <c r="AA19" s="29"/>
+      <c r="AB19" s="29"/>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="29" t="s">
+      <c r="A20" s="30" t="s">
         <v>413</v>
       </c>
-      <c r="B20" s="30">
+      <c r="B20" s="31">
         <v>606.61</v>
       </c>
-      <c r="C20" s="30">
+      <c r="C20" s="31">
         <v>412.29</v>
       </c>
-      <c r="D20" s="30">
+      <c r="D20" s="31">
         <v>480.56</v>
       </c>
-      <c r="E20" s="30">
+      <c r="E20" s="31">
         <v>888.02</v>
       </c>
-      <c r="F20" s="30">
+      <c r="F20" s="31">
         <v>1111.69</v>
       </c>
-      <c r="G20" s="30">
+      <c r="G20" s="31">
         <v>553.57</v>
       </c>
-      <c r="H20" s="30">
+      <c r="H20" s="31">
         <v>544.24</v>
       </c>
-      <c r="I20" s="30">
+      <c r="I20" s="31">
         <v>546.19</v>
       </c>
-      <c r="J20" s="30">
+      <c r="J20" s="31">
         <v>704.2</v>
       </c>
-      <c r="K20" s="30">
+      <c r="K20" s="31">
         <v>289.71</v>
       </c>
-      <c r="L20" s="30">
+      <c r="L20" s="31">
         <v>150.12</v>
       </c>
-      <c r="M20" s="30">
+      <c r="M20" s="31">
         <v>189.55</v>
       </c>
-      <c r="N20" s="31">
+      <c r="N20" s="32">
         <v>61.27</v>
       </c>
-      <c r="O20" s="31">
+      <c r="O20" s="32">
         <v>24.45</v>
       </c>
-      <c r="P20" s="31">
+      <c r="P20" s="32">
         <v>56.03</v>
       </c>
-      <c r="Q20" s="31">
+      <c r="Q20" s="32">
         <v>96.41</v>
       </c>
-      <c r="R20" s="31">
+      <c r="R20" s="32">
         <v>90.75</v>
       </c>
-      <c r="S20" s="30">
+      <c r="S20" s="31">
         <v>636.18</v>
       </c>
-      <c r="T20" s="30">
+      <c r="T20" s="31">
         <v>430.03</v>
       </c>
-      <c r="U20" s="30">
+      <c r="U20" s="31">
         <v>537.69</v>
       </c>
-      <c r="V20" s="30">
+      <c r="V20" s="31">
         <v>258.6</v>
       </c>
-      <c r="W20" s="30">
+      <c r="W20" s="31">
         <v>230.51</v>
       </c>
-      <c r="X20" s="31">
+      <c r="X20" s="32">
         <v>58.43</v>
       </c>
-      <c r="Y20" s="30">
+      <c r="Y20" s="31">
         <v>115.14</v>
       </c>
-      <c r="Z20" s="32"/>
-      <c r="AA20" s="32"/>
-      <c r="AB20" s="32"/>
+      <c r="Z20" s="33"/>
+      <c r="AA20" s="33"/>
+      <c r="AB20" s="33"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="29" t="s">
+      <c r="A21" s="30" t="s">
         <v>414</v>
       </c>
-      <c r="B21" s="30">
+      <c r="B21" s="31">
         <v>699.83</v>
       </c>
-      <c r="C21" s="30">
+      <c r="C21" s="31">
         <v>689.23</v>
       </c>
-      <c r="D21" s="30">
+      <c r="D21" s="31">
         <v>715.62</v>
       </c>
-      <c r="E21" s="30">
+      <c r="E21" s="31">
         <v>728.74</v>
       </c>
-      <c r="F21" s="30">
+      <c r="F21" s="31">
         <v>691.98</v>
       </c>
-      <c r="G21" s="30">
+      <c r="G21" s="31">
         <v>527.58</v>
       </c>
-      <c r="H21" s="30">
+      <c r="H21" s="31">
         <v>446.89</v>
       </c>
-      <c r="I21" s="30">
+      <c r="I21" s="31">
         <v>375.95</v>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="31">
         <v>278.97</v>
       </c>
-      <c r="K21" s="30">
+      <c r="K21" s="31">
         <v>143.02</v>
       </c>
-      <c r="L21" s="31">
+      <c r="L21" s="32">
         <v>96.28</v>
       </c>
-      <c r="M21" s="31">
+      <c r="M21" s="32">
         <v>85.54</v>
       </c>
-      <c r="N21" s="31">
+      <c r="N21" s="32">
         <v>65.78</v>
       </c>
-      <c r="O21" s="30">
+      <c r="O21" s="31">
         <v>180.76</v>
       </c>
-      <c r="P21" s="30">
+      <c r="P21" s="31">
         <v>261.88</v>
       </c>
-      <c r="Q21" s="30">
+      <c r="Q21" s="31">
         <v>358.21</v>
       </c>
-      <c r="R21" s="30">
+      <c r="R21" s="31">
         <v>390.65</v>
       </c>
-      <c r="S21" s="30">
+      <c r="S21" s="31">
         <v>418.6</v>
       </c>
-      <c r="T21" s="30">
+      <c r="T21" s="31">
         <v>303.05</v>
       </c>
-      <c r="U21" s="30">
+      <c r="U21" s="31">
         <v>240.08</v>
       </c>
-      <c r="V21" s="32"/>
-      <c r="W21" s="32"/>
-      <c r="X21" s="32"/>
-      <c r="Y21" s="32"/>
-      <c r="Z21" s="32"/>
-      <c r="AA21" s="32"/>
-      <c r="AB21" s="32"/>
+      <c r="V21" s="33"/>
+      <c r="W21" s="33"/>
+      <c r="X21" s="33"/>
+      <c r="Y21" s="33"/>
+      <c r="Z21" s="33"/>
+      <c r="AA21" s="33"/>
+      <c r="AB21" s="33"/>
     </row>
     <row r="22" ht="15.0" customHeight="1">
-      <c r="A22" s="27" t="s">
+      <c r="A22" s="28" t="s">
         <v>415</v>
       </c>
-      <c r="B22" s="28"/>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
-      <c r="F22" s="28"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="28"/>
-      <c r="K22" s="28"/>
-      <c r="L22" s="28"/>
-      <c r="M22" s="28"/>
-      <c r="N22" s="28"/>
-      <c r="O22" s="28"/>
-      <c r="P22" s="28"/>
-      <c r="Q22" s="28"/>
-      <c r="R22" s="28"/>
-      <c r="S22" s="28"/>
-      <c r="T22" s="28"/>
-      <c r="U22" s="28"/>
-      <c r="V22" s="28"/>
-      <c r="W22" s="28"/>
-      <c r="X22" s="28"/>
-      <c r="Y22" s="28"/>
-      <c r="Z22" s="28"/>
-      <c r="AA22" s="28"/>
-      <c r="AB22" s="28"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="29"/>
+      <c r="F22" s="29"/>
+      <c r="G22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="29"/>
+      <c r="J22" s="29"/>
+      <c r="K22" s="29"/>
+      <c r="L22" s="29"/>
+      <c r="M22" s="29"/>
+      <c r="N22" s="29"/>
+      <c r="O22" s="29"/>
+      <c r="P22" s="29"/>
+      <c r="Q22" s="29"/>
+      <c r="R22" s="29"/>
+      <c r="S22" s="29"/>
+      <c r="T22" s="29"/>
+      <c r="U22" s="29"/>
+      <c r="V22" s="29"/>
+      <c r="W22" s="29"/>
+      <c r="X22" s="29"/>
+      <c r="Y22" s="29"/>
+      <c r="Z22" s="29"/>
+      <c r="AA22" s="29"/>
+      <c r="AB22" s="29"/>
     </row>
     <row r="23" ht="15.0" customHeight="1">
-      <c r="A23" s="29" t="s">
+      <c r="A23" s="30" t="s">
         <v>415</v>
       </c>
-      <c r="B23" s="30">
+      <c r="B23" s="31">
         <v>471.38</v>
       </c>
-      <c r="C23" s="30">
+      <c r="C23" s="31">
         <v>284.35</v>
       </c>
-      <c r="D23" s="30">
+      <c r="D23" s="31">
         <v>367.69</v>
       </c>
-      <c r="E23" s="30">
+      <c r="E23" s="31">
         <v>765.15</v>
       </c>
-      <c r="F23" s="30">
+      <c r="F23" s="31">
         <v>943.97</v>
       </c>
-      <c r="G23" s="30">
+      <c r="G23" s="31">
         <v>551.88</v>
       </c>
-      <c r="H23" s="30">
+      <c r="H23" s="31">
         <v>524.89</v>
       </c>
-      <c r="I23" s="30">
+      <c r="I23" s="31">
         <v>489.94</v>
       </c>
-      <c r="J23" s="30">
+      <c r="J23" s="31">
         <v>634.32</v>
       </c>
-      <c r="K23" s="31">
+      <c r="K23" s="32">
         <v>34.55</v>
       </c>
-      <c r="L23" s="30">
+      <c r="L23" s="31">
         <v>166.66</v>
       </c>
-      <c r="M23" s="30">
+      <c r="M23" s="31">
         <v>209.25</v>
       </c>
-      <c r="N23" s="31">
+      <c r="N23" s="32">
         <v>78.19</v>
       </c>
-      <c r="O23" s="31">
+      <c r="O23" s="32">
         <v>59.23</v>
       </c>
-      <c r="P23" s="31">
+      <c r="P23" s="32">
         <v>81.72</v>
       </c>
-      <c r="Q23" s="30">
+      <c r="Q23" s="31">
         <v>152.06</v>
       </c>
-      <c r="R23" s="31">
+      <c r="R23" s="32">
         <v>90.75</v>
       </c>
-      <c r="S23" s="30">
+      <c r="S23" s="31">
         <v>746.95</v>
       </c>
-      <c r="T23" s="30">
+      <c r="T23" s="31">
         <v>483.31</v>
       </c>
-      <c r="U23" s="30">
+      <c r="U23" s="31">
         <v>582.11</v>
       </c>
-      <c r="V23" s="30">
+      <c r="V23" s="31">
         <v>318.36</v>
       </c>
-      <c r="W23" s="30">
+      <c r="W23" s="31">
         <v>267.42</v>
       </c>
-      <c r="X23" s="30">
+      <c r="X23" s="31">
         <v>105.22</v>
       </c>
-      <c r="Y23" s="30">
+      <c r="Y23" s="31">
         <v>220.96</v>
       </c>
-      <c r="Z23" s="32"/>
-      <c r="AA23" s="32"/>
-      <c r="AB23" s="32"/>
+      <c r="Z23" s="33"/>
+      <c r="AA23" s="33"/>
+      <c r="AB23" s="33"/>
     </row>
     <row r="24" ht="15.0" customHeight="1">
-      <c r="A24" s="29" t="s">
+      <c r="A24" s="30" t="s">
         <v>416</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="31">
         <v>566.51</v>
       </c>
-      <c r="C24" s="30">
+      <c r="C24" s="31">
         <v>582.61</v>
       </c>
-      <c r="D24" s="30">
+      <c r="D24" s="31">
         <v>630.71</v>
       </c>
-      <c r="E24" s="30">
+      <c r="E24" s="31">
         <v>655.17</v>
       </c>
-      <c r="F24" s="30">
+      <c r="F24" s="31">
         <v>629.0</v>
       </c>
-      <c r="G24" s="30">
+      <c r="G24" s="31">
         <v>447.12</v>
       </c>
-      <c r="H24" s="30">
+      <c r="H24" s="31">
         <v>370.07</v>
       </c>
-      <c r="I24" s="30">
+      <c r="I24" s="31">
         <v>306.95</v>
       </c>
-      <c r="J24" s="30">
+      <c r="J24" s="31">
         <v>224.6</v>
       </c>
-      <c r="K24" s="30">
+      <c r="K24" s="31">
         <v>109.58</v>
       </c>
-      <c r="L24" s="30">
+      <c r="L24" s="31">
         <v>119.01</v>
       </c>
-      <c r="M24" s="30">
+      <c r="M24" s="31">
         <v>116.09</v>
       </c>
-      <c r="N24" s="31">
+      <c r="N24" s="32">
         <v>92.39</v>
       </c>
-      <c r="O24" s="30">
+      <c r="O24" s="31">
         <v>226.14</v>
       </c>
-      <c r="P24" s="30">
+      <c r="P24" s="31">
         <v>310.96</v>
       </c>
-      <c r="Q24" s="30">
+      <c r="Q24" s="31">
         <v>411.04</v>
       </c>
-      <c r="R24" s="30">
+      <c r="R24" s="31">
         <v>444.3</v>
       </c>
-      <c r="S24" s="30">
+      <c r="S24" s="31">
         <v>479.63</v>
       </c>
-      <c r="T24" s="30">
+      <c r="T24" s="31">
         <v>351.29</v>
       </c>
-      <c r="U24" s="30">
+      <c r="U24" s="31">
         <v>298.82</v>
       </c>
-      <c r="V24" s="32"/>
-      <c r="W24" s="32"/>
-      <c r="X24" s="32"/>
-      <c r="Y24" s="32"/>
-      <c r="Z24" s="32"/>
-      <c r="AA24" s="32"/>
-      <c r="AB24" s="32"/>
+      <c r="V24" s="33"/>
+      <c r="W24" s="33"/>
+      <c r="X24" s="33"/>
+      <c r="Y24" s="33"/>
+      <c r="Z24" s="33"/>
+      <c r="AA24" s="33"/>
+      <c r="AB24" s="33"/>
     </row>
     <row r="25" ht="15.0" customHeight="1">
-      <c r="A25" s="27" t="s">
+      <c r="A25" s="28" t="s">
         <v>417</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="28"/>
-      <c r="K25" s="28"/>
-      <c r="L25" s="28"/>
-      <c r="M25" s="28"/>
-      <c r="N25" s="28"/>
-      <c r="O25" s="28"/>
-      <c r="P25" s="28"/>
-      <c r="Q25" s="28"/>
-      <c r="R25" s="28"/>
-      <c r="S25" s="28"/>
-      <c r="T25" s="28"/>
-      <c r="U25" s="28"/>
-      <c r="V25" s="28"/>
-      <c r="W25" s="28"/>
-      <c r="X25" s="28"/>
-      <c r="Y25" s="28"/>
-      <c r="Z25" s="28"/>
-      <c r="AA25" s="28"/>
-      <c r="AB25" s="28"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
+      <c r="G25" s="29"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="29"/>
+      <c r="K25" s="29"/>
+      <c r="L25" s="29"/>
+      <c r="M25" s="29"/>
+      <c r="N25" s="29"/>
+      <c r="O25" s="29"/>
+      <c r="P25" s="29"/>
+      <c r="Q25" s="29"/>
+      <c r="R25" s="29"/>
+      <c r="S25" s="29"/>
+      <c r="T25" s="29"/>
+      <c r="U25" s="29"/>
+      <c r="V25" s="29"/>
+      <c r="W25" s="29"/>
+      <c r="X25" s="29"/>
+      <c r="Y25" s="29"/>
+      <c r="Z25" s="29"/>
+      <c r="AA25" s="29"/>
+      <c r="AB25" s="29"/>
     </row>
     <row r="26" ht="15.0" customHeight="1">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="30" t="s">
         <v>418</v>
       </c>
-      <c r="B26" s="31">
+      <c r="B26" s="32">
         <v>13.7</v>
       </c>
-      <c r="C26" s="31">
+      <c r="C26" s="32">
         <v>8.99</v>
       </c>
-      <c r="D26" s="31">
+      <c r="D26" s="32">
         <v>11.5</v>
       </c>
-      <c r="E26" s="31">
+      <c r="E26" s="32">
         <v>36.5</v>
       </c>
-      <c r="F26" s="31">
+      <c r="F26" s="32">
         <v>51.5</v>
       </c>
-      <c r="G26" s="31">
+      <c r="G26" s="32">
         <v>33.9</v>
       </c>
-      <c r="H26" s="31">
+      <c r="H26" s="32">
         <v>33.0</v>
       </c>
-      <c r="I26" s="31">
+      <c r="I26" s="32">
         <v>33.5</v>
       </c>
-      <c r="J26" s="31">
+      <c r="J26" s="32">
         <v>61.9</v>
       </c>
-      <c r="K26" s="31">
+      <c r="K26" s="32">
         <v>33.48</v>
       </c>
-      <c r="L26" s="30">
+      <c r="L26" s="31">
         <v>161.5</v>
       </c>
-      <c r="M26" s="30">
+      <c r="M26" s="31">
         <v>205.81</v>
       </c>
-      <c r="N26" s="31">
+      <c r="N26" s="32">
         <v>83.7</v>
       </c>
-      <c r="O26" s="31">
+      <c r="O26" s="32">
         <v>80.2</v>
       </c>
-      <c r="P26" s="30">
+      <c r="P26" s="31">
         <v>111.13</v>
       </c>
-      <c r="Q26" s="30">
+      <c r="Q26" s="31">
         <v>206.79</v>
       </c>
-      <c r="R26" s="30">
+      <c r="R26" s="31">
         <v>125.62</v>
       </c>
-      <c r="S26" s="30">
+      <c r="S26" s="31">
         <v>1033.96</v>
       </c>
-      <c r="T26" s="30">
+      <c r="T26" s="31">
         <v>1024.39</v>
       </c>
-      <c r="U26" s="30">
+      <c r="U26" s="31">
         <v>1327.37</v>
       </c>
-      <c r="V26" s="30">
+      <c r="V26" s="31">
         <v>990.73</v>
       </c>
-      <c r="W26" s="30">
+      <c r="W26" s="31">
         <v>952.99</v>
       </c>
-      <c r="X26" s="30">
+      <c r="X26" s="31">
         <v>471.78</v>
       </c>
-      <c r="Y26" s="30">
+      <c r="Y26" s="31">
         <v>990.73</v>
       </c>
-      <c r="Z26" s="32"/>
-      <c r="AA26" s="32"/>
-      <c r="AB26" s="32"/>
+      <c r="Z26" s="33"/>
+      <c r="AA26" s="33"/>
+      <c r="AB26" s="33"/>
     </row>
     <row r="27" ht="15.0" customHeight="1">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="30" t="s">
         <v>419</v>
       </c>
-      <c r="B27" s="31">
+      <c r="B27" s="32">
         <v>24.44</v>
       </c>
-      <c r="C27" s="31">
+      <c r="C27" s="32">
         <v>28.48</v>
       </c>
-      <c r="D27" s="31">
+      <c r="D27" s="32">
         <v>33.28</v>
       </c>
-      <c r="E27" s="31">
+      <c r="E27" s="32">
         <v>37.68</v>
       </c>
-      <c r="F27" s="31">
+      <c r="F27" s="32">
         <v>42.76</v>
       </c>
-      <c r="G27" s="31">
+      <c r="G27" s="32">
         <v>39.16</v>
       </c>
-      <c r="H27" s="31">
+      <c r="H27" s="32">
         <v>64.68</v>
       </c>
-      <c r="I27" s="31">
+      <c r="I27" s="32">
         <v>99.24</v>
       </c>
-      <c r="J27" s="30">
+      <c r="J27" s="31">
         <v>109.28</v>
       </c>
-      <c r="K27" s="30">
+      <c r="K27" s="31">
         <v>112.94</v>
       </c>
-      <c r="L27" s="30">
+      <c r="L27" s="31">
         <v>128.47</v>
       </c>
-      <c r="M27" s="30">
+      <c r="M27" s="31">
         <v>137.53</v>
       </c>
-      <c r="N27" s="30">
+      <c r="N27" s="31">
         <v>121.49</v>
       </c>
-      <c r="O27" s="30">
+      <c r="O27" s="31">
         <v>311.54</v>
       </c>
-      <c r="P27" s="30">
+      <c r="P27" s="31">
         <v>500.38</v>
       </c>
-      <c r="Q27" s="30">
+      <c r="Q27" s="31">
         <v>743.63</v>
       </c>
-      <c r="R27" s="30">
+      <c r="R27" s="31">
         <v>900.41</v>
       </c>
-      <c r="S27" s="30">
+      <c r="S27" s="31">
         <v>1065.89</v>
       </c>
-      <c r="T27" s="30">
+      <c r="T27" s="31">
         <v>953.45</v>
       </c>
-      <c r="U27" s="30">
+      <c r="U27" s="31">
         <v>946.72</v>
       </c>
-      <c r="V27" s="32"/>
-      <c r="W27" s="32"/>
-      <c r="X27" s="32"/>
-      <c r="Y27" s="32"/>
-      <c r="Z27" s="32"/>
-      <c r="AA27" s="32"/>
-      <c r="AB27" s="32"/>
+      <c r="V27" s="33"/>
+      <c r="W27" s="33"/>
+      <c r="X27" s="33"/>
+      <c r="Y27" s="33"/>
+      <c r="Z27" s="33"/>
+      <c r="AA27" s="33"/>
+      <c r="AB27" s="33"/>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="27" t="s">
+      <c r="A28" s="28" t="s">
         <v>420</v>
       </c>
-      <c r="B28" s="28"/>
-      <c r="C28" s="28"/>
-      <c r="D28" s="28"/>
-      <c r="E28" s="28"/>
-      <c r="F28" s="28"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="28"/>
-      <c r="K28" s="28"/>
-      <c r="L28" s="28"/>
-      <c r="M28" s="28"/>
-      <c r="N28" s="28"/>
-      <c r="O28" s="28"/>
-      <c r="P28" s="28"/>
-      <c r="Q28" s="28"/>
-      <c r="R28" s="28"/>
-      <c r="S28" s="28"/>
-      <c r="T28" s="28"/>
-      <c r="U28" s="28"/>
-      <c r="V28" s="28"/>
-      <c r="W28" s="28"/>
-      <c r="X28" s="28"/>
-      <c r="Y28" s="28"/>
-      <c r="Z28" s="28"/>
-      <c r="AA28" s="28"/>
-      <c r="AB28" s="28"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="29"/>
+      <c r="F28" s="29"/>
+      <c r="G28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="29"/>
+      <c r="J28" s="29"/>
+      <c r="K28" s="29"/>
+      <c r="L28" s="29"/>
+      <c r="M28" s="29"/>
+      <c r="N28" s="29"/>
+      <c r="O28" s="29"/>
+      <c r="P28" s="29"/>
+      <c r="Q28" s="29"/>
+      <c r="R28" s="29"/>
+      <c r="S28" s="29"/>
+      <c r="T28" s="29"/>
+      <c r="U28" s="29"/>
+      <c r="V28" s="29"/>
+      <c r="W28" s="29"/>
+      <c r="X28" s="29"/>
+      <c r="Y28" s="29"/>
+      <c r="Z28" s="29"/>
+      <c r="AA28" s="29"/>
+      <c r="AB28" s="29"/>
     </row>
     <row r="29" ht="15.0" customHeight="1">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="30" t="s">
         <v>421</v>
       </c>
-      <c r="B29" s="33">
+      <c r="B29" s="34">
         <v>-7.92</v>
       </c>
-      <c r="C29" s="33">
+      <c r="C29" s="34">
         <v>-1.77</v>
       </c>
-      <c r="D29" s="33">
+      <c r="D29" s="34">
         <v>-23.02</v>
       </c>
-      <c r="E29" s="33">
+      <c r="E29" s="34">
         <v>-8.71</v>
       </c>
-      <c r="F29" s="33">
+      <c r="F29" s="34">
         <v>-6.26</v>
       </c>
-      <c r="G29" s="34">
+      <c r="G29" s="35">
         <v>3.62</v>
       </c>
-      <c r="H29" s="34">
+      <c r="H29" s="35">
         <v>3.09</v>
       </c>
-      <c r="I29" s="33">
+      <c r="I29" s="34">
         <v>-8.17</v>
       </c>
-      <c r="J29" s="33">
+      <c r="J29" s="34">
         <v>-8.07</v>
       </c>
-      <c r="K29" s="34">
+      <c r="K29" s="35">
         <v>99.13</v>
       </c>
-      <c r="L29" s="33">
+      <c r="L29" s="34">
         <v>-0.89</v>
       </c>
-      <c r="M29" s="33">
+      <c r="M29" s="34">
         <v>-3.24</v>
       </c>
-      <c r="N29" s="33">
+      <c r="N29" s="34">
         <v>-41.58</v>
       </c>
-      <c r="O29" s="33">
+      <c r="O29" s="34">
         <v>-49.92</v>
       </c>
-      <c r="P29" s="33">
+      <c r="P29" s="34">
         <v>-27.92</v>
       </c>
-      <c r="Q29" s="33">
+      <c r="Q29" s="34">
         <v>-15.83</v>
       </c>
-      <c r="R29" s="33">
+      <c r="R29" s="34">
         <v>-22.87</v>
       </c>
-      <c r="S29" s="33">
+      <c r="S29" s="34">
         <v>-3.61</v>
       </c>
-      <c r="T29" s="33">
+      <c r="T29" s="34">
         <v>-7.37</v>
       </c>
-      <c r="U29" s="33">
+      <c r="U29" s="34">
         <v>-7.42</v>
       </c>
-      <c r="V29" s="33">
+      <c r="V29" s="34">
         <v>-10.29</v>
       </c>
-      <c r="W29" s="33">
+      <c r="W29" s="34">
         <v>-24.29</v>
       </c>
-      <c r="X29" s="33">
+      <c r="X29" s="34">
         <v>-54.32</v>
       </c>
-      <c r="Y29" s="33">
+      <c r="Y29" s="34">
         <v>-29.04</v>
       </c>
-      <c r="Z29" s="34"/>
-      <c r="AA29" s="34"/>
-      <c r="AB29" s="34"/>
+      <c r="Z29" s="35"/>
+      <c r="AA29" s="35"/>
+      <c r="AB29" s="35"/>
     </row>
     <row r="30" ht="15.0" customHeight="1">
-      <c r="A30" s="29" t="s">
+      <c r="A30" s="30" t="s">
         <v>422</v>
       </c>
-      <c r="B30" s="33">
+      <c r="B30" s="34">
         <v>-8.43</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C30" s="34">
         <v>-5.61</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="34">
         <v>-4.09</v>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="34">
         <v>-3.66</v>
       </c>
-      <c r="F30" s="33">
+      <c r="F30" s="34">
         <v>-4.07</v>
       </c>
-      <c r="G30" s="34">
+      <c r="G30" s="35">
         <v>14.15</v>
       </c>
-      <c r="H30" s="34">
+      <c r="H30" s="35">
         <v>7.74</v>
       </c>
-      <c r="I30" s="34">
+      <c r="I30" s="35">
         <v>3.5</v>
       </c>
-      <c r="J30" s="33">
+      <c r="J30" s="34">
         <v>-2.69</v>
       </c>
-      <c r="K30" s="33">
+      <c r="K30" s="34">
         <v>-8.81</v>
       </c>
-      <c r="L30" s="33">
+      <c r="L30" s="34">
         <v>-17.74</v>
       </c>
-      <c r="M30" s="33">
+      <c r="M30" s="34">
         <v>-21.13</v>
       </c>
-      <c r="N30" s="33">
+      <c r="N30" s="34">
         <v>-27.55</v>
       </c>
-      <c r="O30" s="33">
+      <c r="O30" s="34">
         <v>-10.91</v>
       </c>
-      <c r="P30" s="33">
+      <c r="P30" s="34">
         <v>-8.21</v>
       </c>
-      <c r="Q30" s="33">
+      <c r="Q30" s="34">
         <v>-7.34</v>
       </c>
-      <c r="R30" s="33">
+      <c r="R30" s="34">
         <v>-7.6</v>
       </c>
-      <c r="S30" s="33">
+      <c r="S30" s="34">
         <v>-10.22</v>
       </c>
-      <c r="T30" s="33">
+      <c r="T30" s="34">
         <v>-16.02</v>
       </c>
-      <c r="U30" s="33">
+      <c r="U30" s="34">
         <v>-20.62</v>
       </c>
-      <c r="V30" s="34"/>
-      <c r="W30" s="34"/>
-      <c r="X30" s="34"/>
-      <c r="Y30" s="34"/>
-      <c r="Z30" s="34"/>
-      <c r="AA30" s="34"/>
-      <c r="AB30" s="34"/>
+      <c r="V30" s="35"/>
+      <c r="W30" s="35"/>
+      <c r="X30" s="35"/>
+      <c r="Y30" s="35"/>
+      <c r="Z30" s="35"/>
+      <c r="AA30" s="35"/>
+      <c r="AB30" s="35"/>
     </row>
     <row r="31" ht="15.0" customHeight="1">
-      <c r="A31" s="27" t="s">
+      <c r="A31" s="28" t="s">
         <v>423</v>
       </c>
-      <c r="B31" s="28"/>
-      <c r="C31" s="28"/>
-      <c r="D31" s="28"/>
-      <c r="E31" s="28"/>
-      <c r="F31" s="28"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="28"/>
-      <c r="K31" s="28"/>
-      <c r="L31" s="28"/>
-      <c r="M31" s="28"/>
-      <c r="N31" s="28"/>
-      <c r="O31" s="28"/>
-      <c r="P31" s="28"/>
-      <c r="Q31" s="28"/>
-      <c r="R31" s="28"/>
-      <c r="S31" s="28"/>
-      <c r="T31" s="28"/>
-      <c r="U31" s="28"/>
-      <c r="V31" s="28"/>
-      <c r="W31" s="28"/>
-      <c r="X31" s="28"/>
-      <c r="Y31" s="28"/>
-      <c r="Z31" s="28"/>
-      <c r="AA31" s="28"/>
-      <c r="AB31" s="28"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="29"/>
+      <c r="F31" s="29"/>
+      <c r="G31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="29"/>
+      <c r="J31" s="29"/>
+      <c r="K31" s="29"/>
+      <c r="L31" s="29"/>
+      <c r="M31" s="29"/>
+      <c r="N31" s="29"/>
+      <c r="O31" s="29"/>
+      <c r="P31" s="29"/>
+      <c r="Q31" s="29"/>
+      <c r="R31" s="29"/>
+      <c r="S31" s="29"/>
+      <c r="T31" s="29"/>
+      <c r="U31" s="29"/>
+      <c r="V31" s="29"/>
+      <c r="W31" s="29"/>
+      <c r="X31" s="29"/>
+      <c r="Y31" s="29"/>
+      <c r="Z31" s="29"/>
+      <c r="AA31" s="29"/>
+      <c r="AB31" s="29"/>
     </row>
     <row r="32" ht="15.0" customHeight="1">
-      <c r="A32" s="29" t="s">
+      <c r="A32" s="30" t="s">
         <v>424</v>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="32">
         <v>0.83</v>
       </c>
-      <c r="C32" s="31">
+      <c r="C32" s="32">
         <v>0.5</v>
       </c>
-      <c r="D32" s="31">
+      <c r="D32" s="32">
         <v>0.61</v>
       </c>
-      <c r="E32" s="31">
+      <c r="E32" s="32">
         <v>1.38</v>
       </c>
-      <c r="F32" s="31">
+      <c r="F32" s="32">
         <v>1.68</v>
       </c>
-      <c r="G32" s="31">
+      <c r="G32" s="32">
         <v>1.21</v>
       </c>
-      <c r="H32" s="31">
+      <c r="H32" s="32">
         <v>1.02</v>
       </c>
-      <c r="I32" s="31">
+      <c r="I32" s="32">
         <v>1.09</v>
       </c>
-      <c r="J32" s="31">
+      <c r="J32" s="32">
         <v>2.7</v>
       </c>
-      <c r="K32" s="31">
+      <c r="K32" s="32">
         <v>0.82</v>
       </c>
-      <c r="L32" s="31">
+      <c r="L32" s="32">
         <v>2.52</v>
       </c>
-      <c r="M32" s="31">
+      <c r="M32" s="32">
         <v>2.95</v>
       </c>
-      <c r="N32" s="31">
+      <c r="N32" s="32">
         <v>1.33</v>
       </c>
-      <c r="O32" s="31">
+      <c r="O32" s="32">
         <v>0.73</v>
       </c>
-      <c r="P32" s="31">
+      <c r="P32" s="32">
         <v>0.69</v>
       </c>
-      <c r="Q32" s="31">
+      <c r="Q32" s="32">
         <v>0.88</v>
       </c>
-      <c r="R32" s="31">
+      <c r="R32" s="32">
         <v>0.44</v>
       </c>
-      <c r="S32" s="31">
+      <c r="S32" s="32">
         <v>1.82</v>
       </c>
-      <c r="T32" s="31">
+      <c r="T32" s="32">
         <v>2.85</v>
       </c>
-      <c r="U32" s="31">
+      <c r="U32" s="32">
         <v>3.64</v>
       </c>
-      <c r="V32" s="31">
+      <c r="V32" s="32">
         <v>2.9</v>
       </c>
-      <c r="W32" s="31">
+      <c r="W32" s="32">
         <v>5.04</v>
       </c>
-      <c r="X32" s="31">
+      <c r="X32" s="32">
         <v>1.62</v>
       </c>
-      <c r="Y32" s="31">
+      <c r="Y32" s="32">
         <v>1.63</v>
       </c>
-      <c r="Z32" s="32"/>
-      <c r="AA32" s="32"/>
-      <c r="AB32" s="32"/>
+      <c r="Z32" s="33"/>
+      <c r="AA32" s="33"/>
+      <c r="AB32" s="33"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
-      <c r="A33" s="29" t="s">
+      <c r="A33" s="30" t="s">
         <v>425</v>
       </c>
-      <c r="B33" s="31">
+      <c r="B33" s="32">
         <v>1.1</v>
       </c>
-      <c r="C33" s="31">
+      <c r="C33" s="32">
         <v>1.17</v>
       </c>
-      <c r="D33" s="31">
+      <c r="D33" s="32">
         <v>1.22</v>
       </c>
-      <c r="E33" s="31">
+      <c r="E33" s="32">
         <v>1.27</v>
       </c>
-      <c r="F33" s="31">
+      <c r="F33" s="32">
         <v>1.48</v>
       </c>
-      <c r="G33" s="31">
+      <c r="G33" s="32">
         <v>1.26</v>
       </c>
-      <c r="H33" s="31">
+      <c r="H33" s="32">
         <v>1.69</v>
       </c>
-      <c r="I33" s="31">
+      <c r="I33" s="32">
         <v>2.17</v>
       </c>
-      <c r="J33" s="31">
+      <c r="J33" s="32">
         <v>2.1</v>
       </c>
-      <c r="K33" s="31">
+      <c r="K33" s="32">
         <v>1.63</v>
       </c>
-      <c r="L33" s="31">
+      <c r="L33" s="32">
         <v>1.38</v>
       </c>
-      <c r="M33" s="31">
+      <c r="M33" s="32">
         <v>1.08</v>
       </c>
-      <c r="N33" s="31">
+      <c r="N33" s="32">
         <v>0.71</v>
       </c>
-      <c r="O33" s="31">
+      <c r="O33" s="32">
         <v>1.14</v>
       </c>
-      <c r="P33" s="31">
+      <c r="P33" s="32">
         <v>1.55</v>
       </c>
-      <c r="Q33" s="31">
+      <c r="Q33" s="32">
         <v>2.05</v>
       </c>
-      <c r="R33" s="31">
+      <c r="R33" s="32">
         <v>2.34</v>
       </c>
-      <c r="S33" s="31">
+      <c r="S33" s="32">
         <v>2.92</v>
       </c>
-      <c r="T33" s="31">
+      <c r="T33" s="32">
         <v>3.08</v>
       </c>
-      <c r="U33" s="31">
+      <c r="U33" s="32">
         <v>2.64</v>
       </c>
-      <c r="V33" s="32"/>
-      <c r="W33" s="32"/>
-      <c r="X33" s="32"/>
-      <c r="Y33" s="32"/>
-      <c r="Z33" s="32"/>
-      <c r="AA33" s="32"/>
-      <c r="AB33" s="32"/>
+      <c r="V33" s="33"/>
+      <c r="W33" s="33"/>
+      <c r="X33" s="33"/>
+      <c r="Y33" s="33"/>
+      <c r="Z33" s="33"/>
+      <c r="AA33" s="33"/>
+      <c r="AB33" s="33"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="27" t="s">
+      <c r="A34" s="28" t="s">
         <v>426</v>
       </c>
-      <c r="B34" s="28"/>
-      <c r="C34" s="28"/>
-      <c r="D34" s="28"/>
-      <c r="E34" s="28"/>
-      <c r="F34" s="28"/>
-      <c r="G34" s="28"/>
-      <c r="H34" s="28"/>
-      <c r="I34" s="28"/>
-      <c r="J34" s="28"/>
-      <c r="K34" s="28"/>
-      <c r="L34" s="28"/>
-      <c r="M34" s="28"/>
-      <c r="N34" s="28"/>
-      <c r="O34" s="28"/>
-      <c r="P34" s="28"/>
-      <c r="Q34" s="28"/>
-      <c r="R34" s="28"/>
-      <c r="S34" s="28"/>
-      <c r="T34" s="28"/>
-      <c r="U34" s="28"/>
-      <c r="V34" s="28"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="28"/>
-      <c r="Z34" s="28"/>
-      <c r="AA34" s="28"/>
-      <c r="AB34" s="28"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="29"/>
+      <c r="F34" s="29"/>
+      <c r="G34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+      <c r="J34" s="29"/>
+      <c r="K34" s="29"/>
+      <c r="L34" s="29"/>
+      <c r="M34" s="29"/>
+      <c r="N34" s="29"/>
+      <c r="O34" s="29"/>
+      <c r="P34" s="29"/>
+      <c r="Q34" s="29"/>
+      <c r="R34" s="29"/>
+      <c r="S34" s="29"/>
+      <c r="T34" s="29"/>
+      <c r="U34" s="29"/>
+      <c r="V34" s="29"/>
+      <c r="W34" s="29"/>
+      <c r="X34" s="29"/>
+      <c r="Y34" s="29"/>
+      <c r="Z34" s="29"/>
+      <c r="AA34" s="29"/>
+      <c r="AB34" s="29"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="29" t="s">
+      <c r="A35" s="30" t="s">
         <v>427</v>
       </c>
-      <c r="B35" s="32"/>
-      <c r="C35" s="32"/>
-      <c r="D35" s="32"/>
-      <c r="E35" s="32"/>
-      <c r="F35" s="32"/>
-      <c r="G35" s="32"/>
-      <c r="H35" s="32"/>
-      <c r="I35" s="32"/>
-      <c r="J35" s="32"/>
-      <c r="K35" s="32"/>
-      <c r="L35" s="31">
+      <c r="B35" s="33"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="33"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="33"/>
+      <c r="J35" s="33"/>
+      <c r="K35" s="33"/>
+      <c r="L35" s="32">
         <v>9.39</v>
       </c>
-      <c r="M35" s="31">
+      <c r="M35" s="32">
         <v>9.35</v>
       </c>
-      <c r="N35" s="31">
+      <c r="N35" s="32">
         <v>9.91</v>
       </c>
-      <c r="O35" s="31">
+      <c r="O35" s="32">
         <v>2.86</v>
       </c>
-      <c r="P35" s="31">
+      <c r="P35" s="32">
         <v>1.27</v>
       </c>
-      <c r="Q35" s="31">
+      <c r="Q35" s="32">
         <v>2.78</v>
       </c>
-      <c r="R35" s="31">
+      <c r="R35" s="32">
         <v>1.38</v>
       </c>
-      <c r="S35" s="31">
+      <c r="S35" s="32">
         <v>8.32</v>
       </c>
-      <c r="T35" s="31">
+      <c r="T35" s="32">
         <v>6.53</v>
       </c>
-      <c r="U35" s="31">
+      <c r="U35" s="32">
         <v>9.12</v>
       </c>
-      <c r="V35" s="31">
+      <c r="V35" s="32">
         <v>3.23</v>
       </c>
-      <c r="W35" s="31">
+      <c r="W35" s="32">
         <v>5.65</v>
       </c>
-      <c r="X35" s="31">
+      <c r="X35" s="32">
         <v>1.91</v>
       </c>
-      <c r="Y35" s="31">
+      <c r="Y35" s="32">
         <v>1.84</v>
       </c>
-      <c r="Z35" s="32"/>
-      <c r="AA35" s="32"/>
-      <c r="AB35" s="32"/>
+      <c r="Z35" s="33"/>
+      <c r="AA35" s="33"/>
+      <c r="AB35" s="33"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="29" t="s">
+      <c r="A36" s="30" t="s">
         <v>428</v>
       </c>
-      <c r="B36" s="32"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="32"/>
-      <c r="E36" s="32"/>
-      <c r="F36" s="32"/>
-      <c r="G36" s="32"/>
-      <c r="H36" s="32"/>
-      <c r="I36" s="32"/>
-      <c r="J36" s="32"/>
-      <c r="K36" s="32"/>
-      <c r="L36" s="31">
+      <c r="B36" s="33"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="33"/>
+      <c r="E36" s="33"/>
+      <c r="F36" s="33"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="33"/>
+      <c r="I36" s="33"/>
+      <c r="J36" s="33"/>
+      <c r="K36" s="33"/>
+      <c r="L36" s="32">
         <v>3.93</v>
       </c>
-      <c r="M36" s="31">
+      <c r="M36" s="32">
         <v>3.12</v>
       </c>
-      <c r="N36" s="31">
+      <c r="N36" s="32">
         <v>2.1</v>
       </c>
-      <c r="O36" s="31">
+      <c r="O36" s="32">
         <v>3.84</v>
       </c>
-      <c r="P36" s="31">
+      <c r="P36" s="32">
         <v>4.68</v>
       </c>
-      <c r="Q36" s="31">
+      <c r="Q36" s="32">
         <v>6.28</v>
       </c>
-      <c r="R36" s="31">
+      <c r="R36" s="32">
         <v>5.46</v>
       </c>
-      <c r="S36" s="31">
+      <c r="S36" s="32">
         <v>5.91</v>
       </c>
-      <c r="T36" s="31">
+      <c r="T36" s="32">
         <v>4.65</v>
       </c>
-      <c r="U36" s="31">
+      <c r="U36" s="32">
         <v>3.37</v>
       </c>
-      <c r="V36" s="32"/>
-      <c r="W36" s="32"/>
-      <c r="X36" s="32"/>
-      <c r="Y36" s="32"/>
-      <c r="Z36" s="32"/>
-      <c r="AA36" s="32"/>
-      <c r="AB36" s="32"/>
+      <c r="V36" s="33"/>
+      <c r="W36" s="33"/>
+      <c r="X36" s="33"/>
+      <c r="Y36" s="33"/>
+      <c r="Z36" s="33"/>
+      <c r="AA36" s="33"/>
+      <c r="AB36" s="33"/>
     </row>
     <row r="37" ht="15.0" customHeight="1">
-      <c r="A37" s="27" t="s">
+      <c r="A37" s="28" t="s">
         <v>429</v>
       </c>
-      <c r="B37" s="28"/>
-      <c r="C37" s="28"/>
-      <c r="D37" s="28"/>
-      <c r="E37" s="28"/>
-      <c r="F37" s="28"/>
-      <c r="G37" s="28"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="28"/>
-      <c r="J37" s="28"/>
-      <c r="K37" s="28"/>
-      <c r="L37" s="28"/>
-      <c r="M37" s="28"/>
-      <c r="N37" s="28"/>
-      <c r="O37" s="28"/>
-      <c r="P37" s="28"/>
-      <c r="Q37" s="28"/>
-      <c r="R37" s="28"/>
-      <c r="S37" s="28"/>
-      <c r="T37" s="28"/>
-      <c r="U37" s="28"/>
-      <c r="V37" s="28"/>
-      <c r="W37" s="28"/>
-      <c r="X37" s="28"/>
-      <c r="Y37" s="28"/>
-      <c r="Z37" s="28"/>
-      <c r="AA37" s="28"/>
-      <c r="AB37" s="28"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="29"/>
+      <c r="F37" s="29"/>
+      <c r="G37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="29"/>
+      <c r="J37" s="29"/>
+      <c r="K37" s="29"/>
+      <c r="L37" s="29"/>
+      <c r="M37" s="29"/>
+      <c r="N37" s="29"/>
+      <c r="O37" s="29"/>
+      <c r="P37" s="29"/>
+      <c r="Q37" s="29"/>
+      <c r="R37" s="29"/>
+      <c r="S37" s="29"/>
+      <c r="T37" s="29"/>
+      <c r="U37" s="29"/>
+      <c r="V37" s="29"/>
+      <c r="W37" s="29"/>
+      <c r="X37" s="29"/>
+      <c r="Y37" s="29"/>
+      <c r="Z37" s="29"/>
+      <c r="AA37" s="29"/>
+      <c r="AB37" s="29"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="29" t="s">
+      <c r="A38" s="30" t="s">
         <v>430</v>
       </c>
-      <c r="B38" s="31">
+      <c r="B38" s="32">
         <v>0.41</v>
       </c>
-      <c r="C38" s="31">
+      <c r="C38" s="32">
         <v>0.26</v>
       </c>
-      <c r="D38" s="31">
+      <c r="D38" s="32">
         <v>0.21</v>
       </c>
-      <c r="E38" s="31">
+      <c r="E38" s="32">
         <v>0.53</v>
       </c>
-      <c r="F38" s="31">
+      <c r="F38" s="32">
         <v>0.82</v>
       </c>
-      <c r="G38" s="31">
+      <c r="G38" s="32">
         <v>0.48</v>
       </c>
-      <c r="H38" s="31">
+      <c r="H38" s="32">
         <v>0.48</v>
       </c>
-      <c r="I38" s="31">
+      <c r="I38" s="32">
         <v>0.58</v>
       </c>
-      <c r="J38" s="31">
+      <c r="J38" s="32">
         <v>0.68</v>
       </c>
-      <c r="K38" s="31">
+      <c r="K38" s="32">
         <v>0.05</v>
       </c>
-      <c r="L38" s="31">
+      <c r="L38" s="32">
         <v>3.24</v>
       </c>
-      <c r="M38" s="31">
+      <c r="M38" s="32">
         <v>4.04</v>
       </c>
-      <c r="N38" s="31">
+      <c r="N38" s="32">
         <v>1.77</v>
       </c>
-      <c r="O38" s="31">
+      <c r="O38" s="32">
         <v>1.16</v>
       </c>
-      <c r="P38" s="31">
+      <c r="P38" s="32">
         <v>1.53</v>
       </c>
-      <c r="Q38" s="31">
+      <c r="Q38" s="32">
         <v>2.36</v>
       </c>
-      <c r="R38" s="31">
+      <c r="R38" s="32">
         <v>0.91</v>
       </c>
-      <c r="S38" s="31">
+      <c r="S38" s="32">
         <v>6.52</v>
       </c>
-      <c r="T38" s="31">
+      <c r="T38" s="32">
         <v>9.32</v>
       </c>
-      <c r="U38" s="31">
+      <c r="U38" s="32">
         <v>12.82</v>
       </c>
-      <c r="V38" s="31">
+      <c r="V38" s="32">
         <v>5.66</v>
       </c>
-      <c r="W38" s="31">
+      <c r="W38" s="32">
         <v>9.4</v>
       </c>
-      <c r="X38" s="31">
+      <c r="X38" s="32">
         <v>3.63</v>
       </c>
-      <c r="Y38" s="31">
+      <c r="Y38" s="32">
         <v>52.71</v>
       </c>
-      <c r="Z38" s="32"/>
-      <c r="AA38" s="32"/>
-      <c r="AB38" s="32"/>
+      <c r="Z38" s="33"/>
+      <c r="AA38" s="33"/>
+      <c r="AB38" s="33"/>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="29" t="s">
+      <c r="A39" s="30" t="s">
         <v>431</v>
       </c>
-      <c r="B39" s="31">
+      <c r="B39" s="32">
         <v>0.48</v>
       </c>
-      <c r="C39" s="31">
+      <c r="C39" s="32">
         <v>0.48</v>
       </c>
-      <c r="D39" s="31">
+      <c r="D39" s="32">
         <v>0.51</v>
       </c>
-      <c r="E39" s="31">
+      <c r="E39" s="32">
         <v>0.57</v>
       </c>
-      <c r="F39" s="31">
+      <c r="F39" s="32">
         <v>0.61</v>
       </c>
-      <c r="G39" s="31">
+      <c r="G39" s="32">
         <v>0.22</v>
       </c>
-      <c r="H39" s="31">
+      <c r="H39" s="32">
         <v>0.37</v>
       </c>
-      <c r="I39" s="31">
+      <c r="I39" s="32">
         <v>0.58</v>
       </c>
-      <c r="J39" s="31">
+      <c r="J39" s="32">
         <v>0.64</v>
       </c>
-      <c r="K39" s="31">
+      <c r="K39" s="32">
         <v>0.68</v>
       </c>
-      <c r="L39" s="31">
+      <c r="L39" s="32">
         <v>2.21</v>
       </c>
-      <c r="M39" s="31">
+      <c r="M39" s="32">
         <v>2.1</v>
       </c>
-      <c r="N39" s="31">
+      <c r="N39" s="32">
         <v>1.47</v>
       </c>
-      <c r="O39" s="31">
+      <c r="O39" s="32">
         <v>2.96</v>
       </c>
-      <c r="P39" s="31">
+      <c r="P39" s="32">
         <v>4.42</v>
       </c>
-      <c r="Q39" s="31">
+      <c r="Q39" s="32">
         <v>6.23</v>
       </c>
-      <c r="R39" s="31">
+      <c r="R39" s="32">
         <v>6.58</v>
       </c>
-      <c r="S39" s="31">
+      <c r="S39" s="32">
         <v>8.22</v>
       </c>
-      <c r="T39" s="31">
+      <c r="T39" s="32">
         <v>7.69</v>
       </c>
-      <c r="U39" s="31">
+      <c r="U39" s="32">
         <v>8.95</v>
       </c>
-      <c r="V39" s="32"/>
-      <c r="W39" s="32"/>
-      <c r="X39" s="32"/>
-      <c r="Y39" s="32"/>
-      <c r="Z39" s="32"/>
-      <c r="AA39" s="32"/>
-      <c r="AB39" s="32"/>
+      <c r="V39" s="33"/>
+      <c r="W39" s="33"/>
+      <c r="X39" s="33"/>
+      <c r="Y39" s="33"/>
+      <c r="Z39" s="33"/>
+      <c r="AA39" s="33"/>
+      <c r="AB39" s="33"/>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="27" t="s">
+      <c r="A40" s="28" t="s">
         <v>432</v>
       </c>
-      <c r="B40" s="28"/>
-      <c r="C40" s="28"/>
-      <c r="D40" s="28"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="28"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="28"/>
-      <c r="J40" s="28"/>
-      <c r="K40" s="28"/>
-      <c r="L40" s="28"/>
-      <c r="M40" s="28"/>
-      <c r="N40" s="28"/>
-      <c r="O40" s="28"/>
-      <c r="P40" s="28"/>
-      <c r="Q40" s="28"/>
-      <c r="R40" s="28"/>
-      <c r="S40" s="28"/>
-      <c r="T40" s="28"/>
-      <c r="U40" s="28"/>
-      <c r="V40" s="28"/>
-      <c r="W40" s="28"/>
-      <c r="X40" s="28"/>
-      <c r="Y40" s="28"/>
-      <c r="Z40" s="28"/>
-      <c r="AA40" s="28"/>
-      <c r="AB40" s="28"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="29"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="29"/>
+      <c r="K40" s="29"/>
+      <c r="L40" s="29"/>
+      <c r="M40" s="29"/>
+      <c r="N40" s="29"/>
+      <c r="O40" s="29"/>
+      <c r="P40" s="29"/>
+      <c r="Q40" s="29"/>
+      <c r="R40" s="29"/>
+      <c r="S40" s="29"/>
+      <c r="T40" s="29"/>
+      <c r="U40" s="29"/>
+      <c r="V40" s="29"/>
+      <c r="W40" s="29"/>
+      <c r="X40" s="29"/>
+      <c r="Y40" s="29"/>
+      <c r="Z40" s="29"/>
+      <c r="AA40" s="29"/>
+      <c r="AB40" s="29"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="29" t="s">
+      <c r="A41" s="30" t="s">
         <v>433</v>
       </c>
-      <c r="B41" s="32"/>
-      <c r="C41" s="32"/>
-      <c r="D41" s="32"/>
-      <c r="E41" s="32"/>
-      <c r="F41" s="32"/>
-      <c r="G41" s="31">
+      <c r="B41" s="33"/>
+      <c r="C41" s="33"/>
+      <c r="D41" s="33"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="33"/>
+      <c r="G41" s="32">
         <v>27.59</v>
       </c>
-      <c r="H41" s="31">
+      <c r="H41" s="32">
         <v>32.36</v>
       </c>
-      <c r="I41" s="32"/>
-      <c r="J41" s="32"/>
-      <c r="K41" s="31">
+      <c r="I41" s="33"/>
+      <c r="J41" s="33"/>
+      <c r="K41" s="32">
         <v>1.01</v>
       </c>
-      <c r="L41" s="32"/>
-      <c r="M41" s="32"/>
-      <c r="N41" s="32"/>
-      <c r="O41" s="32"/>
-      <c r="P41" s="32"/>
-      <c r="Q41" s="32"/>
-      <c r="R41" s="32"/>
-      <c r="S41" s="32"/>
-      <c r="T41" s="32"/>
-      <c r="U41" s="32"/>
-      <c r="V41" s="32"/>
-      <c r="W41" s="32"/>
-      <c r="X41" s="32"/>
-      <c r="Y41" s="32"/>
-      <c r="Z41" s="32"/>
-      <c r="AA41" s="32"/>
-      <c r="AB41" s="32"/>
+      <c r="L41" s="33"/>
+      <c r="M41" s="33"/>
+      <c r="N41" s="33"/>
+      <c r="O41" s="33"/>
+      <c r="P41" s="33"/>
+      <c r="Q41" s="33"/>
+      <c r="R41" s="33"/>
+      <c r="S41" s="33"/>
+      <c r="T41" s="33"/>
+      <c r="U41" s="33"/>
+      <c r="V41" s="33"/>
+      <c r="W41" s="33"/>
+      <c r="X41" s="33"/>
+      <c r="Y41" s="33"/>
+      <c r="Z41" s="33"/>
+      <c r="AA41" s="33"/>
+      <c r="AB41" s="33"/>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="29" t="s">
+      <c r="A42" s="30" t="s">
         <v>434</v>
       </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="31">
+      <c r="B42" s="33"/>
+      <c r="C42" s="33"/>
+      <c r="D42" s="33"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="33"/>
+      <c r="G42" s="32">
         <v>7.07</v>
       </c>
-      <c r="H42" s="31">
+      <c r="H42" s="32">
         <v>12.91</v>
       </c>
-      <c r="I42" s="31">
+      <c r="I42" s="32">
         <v>28.58</v>
       </c>
-      <c r="J42" s="32"/>
-      <c r="K42" s="32"/>
-      <c r="L42" s="32"/>
-      <c r="M42" s="32"/>
-      <c r="N42" s="32"/>
-      <c r="O42" s="32"/>
-      <c r="P42" s="32"/>
-      <c r="Q42" s="32"/>
-      <c r="R42" s="32"/>
-      <c r="S42" s="32"/>
-      <c r="T42" s="32"/>
-      <c r="U42" s="32"/>
-      <c r="V42" s="32"/>
-      <c r="W42" s="32"/>
-      <c r="X42" s="32"/>
-      <c r="Y42" s="32"/>
-      <c r="Z42" s="32"/>
-      <c r="AA42" s="32"/>
-      <c r="AB42" s="32"/>
+      <c r="J42" s="33"/>
+      <c r="K42" s="33"/>
+      <c r="L42" s="33"/>
+      <c r="M42" s="33"/>
+      <c r="N42" s="33"/>
+      <c r="O42" s="33"/>
+      <c r="P42" s="33"/>
+      <c r="Q42" s="33"/>
+      <c r="R42" s="33"/>
+      <c r="S42" s="33"/>
+      <c r="T42" s="33"/>
+      <c r="U42" s="33"/>
+      <c r="V42" s="33"/>
+      <c r="W42" s="33"/>
+      <c r="X42" s="33"/>
+      <c r="Y42" s="33"/>
+      <c r="Z42" s="33"/>
+      <c r="AA42" s="33"/>
+      <c r="AB42" s="33"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="27" t="s">
+      <c r="A43" s="28" t="s">
         <v>435</v>
       </c>
-      <c r="B43" s="28"/>
-      <c r="C43" s="28"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="28"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="28"/>
-      <c r="I43" s="28"/>
-      <c r="J43" s="28"/>
-      <c r="K43" s="28"/>
-      <c r="L43" s="28"/>
-      <c r="M43" s="28"/>
-      <c r="N43" s="28"/>
-      <c r="O43" s="28"/>
-      <c r="P43" s="28"/>
-      <c r="Q43" s="28"/>
-      <c r="R43" s="28"/>
-      <c r="S43" s="28"/>
-      <c r="T43" s="28"/>
-      <c r="U43" s="28"/>
-      <c r="V43" s="28"/>
-      <c r="W43" s="28"/>
-      <c r="X43" s="28"/>
-      <c r="Y43" s="28"/>
-      <c r="Z43" s="28"/>
-      <c r="AA43" s="28"/>
-      <c r="AB43" s="28"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="29"/>
+      <c r="F43" s="29"/>
+      <c r="G43" s="29"/>
+      <c r="H43" s="29"/>
+      <c r="I43" s="29"/>
+      <c r="J43" s="29"/>
+      <c r="K43" s="29"/>
+      <c r="L43" s="29"/>
+      <c r="M43" s="29"/>
+      <c r="N43" s="29"/>
+      <c r="O43" s="29"/>
+      <c r="P43" s="29"/>
+      <c r="Q43" s="29"/>
+      <c r="R43" s="29"/>
+      <c r="S43" s="29"/>
+      <c r="T43" s="29"/>
+      <c r="U43" s="29"/>
+      <c r="V43" s="29"/>
+      <c r="W43" s="29"/>
+      <c r="X43" s="29"/>
+      <c r="Y43" s="29"/>
+      <c r="Z43" s="29"/>
+      <c r="AA43" s="29"/>
+      <c r="AB43" s="29"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="29" t="s">
+      <c r="A44" s="30" t="s">
         <v>436</v>
       </c>
-      <c r="B44" s="31">
+      <c r="B44" s="32">
         <v>3.21</v>
       </c>
-      <c r="C44" s="31">
+      <c r="C44" s="32">
         <v>2.19</v>
       </c>
-      <c r="D44" s="31">
+      <c r="D44" s="32">
         <v>2.65</v>
       </c>
-      <c r="E44" s="31">
+      <c r="E44" s="32">
         <v>11.42</v>
       </c>
-      <c r="F44" s="31">
+      <c r="F44" s="32">
         <v>10.26</v>
       </c>
-      <c r="G44" s="32"/>
-      <c r="H44" s="31">
+      <c r="G44" s="33"/>
+      <c r="H44" s="32">
         <v>12.07</v>
       </c>
-      <c r="I44" s="32"/>
-      <c r="J44" s="32"/>
-      <c r="K44" s="31">
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
+      <c r="K44" s="32">
         <v>2.17</v>
       </c>
-      <c r="L44" s="32"/>
-      <c r="M44" s="32"/>
-      <c r="N44" s="32"/>
-      <c r="O44" s="32"/>
-      <c r="P44" s="32"/>
-      <c r="Q44" s="32"/>
-      <c r="R44" s="32"/>
-      <c r="S44" s="32"/>
-      <c r="T44" s="32"/>
-      <c r="U44" s="32"/>
-      <c r="V44" s="32"/>
-      <c r="W44" s="32"/>
-      <c r="X44" s="32"/>
-      <c r="Y44" s="32"/>
-      <c r="Z44" s="32"/>
-      <c r="AA44" s="32"/>
-      <c r="AB44" s="32"/>
+      <c r="L44" s="33"/>
+      <c r="M44" s="33"/>
+      <c r="N44" s="33"/>
+      <c r="O44" s="33"/>
+      <c r="P44" s="33"/>
+      <c r="Q44" s="33"/>
+      <c r="R44" s="33"/>
+      <c r="S44" s="33"/>
+      <c r="T44" s="33"/>
+      <c r="U44" s="33"/>
+      <c r="V44" s="33"/>
+      <c r="W44" s="33"/>
+      <c r="X44" s="33"/>
+      <c r="Y44" s="33"/>
+      <c r="Z44" s="33"/>
+      <c r="AA44" s="33"/>
+      <c r="AB44" s="33"/>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="29" t="s">
+      <c r="A45" s="30" t="s">
         <v>437</v>
       </c>
-      <c r="B45" s="31">
+      <c r="B45" s="32">
         <v>5.84</v>
       </c>
-      <c r="C45" s="31">
+      <c r="C45" s="32">
         <v>9.52</v>
       </c>
-      <c r="D45" s="31">
+      <c r="D45" s="32">
         <v>12.24</v>
       </c>
-      <c r="E45" s="31">
+      <c r="E45" s="32">
         <v>25.44</v>
       </c>
-      <c r="F45" s="30">
+      <c r="F45" s="31">
         <v>859.49</v>
       </c>
-      <c r="G45" s="31">
+      <c r="G45" s="32">
         <v>18.36</v>
       </c>
-      <c r="H45" s="31">
+      <c r="H45" s="32">
         <v>66.36</v>
       </c>
-      <c r="I45" s="32"/>
-      <c r="J45" s="32"/>
-      <c r="K45" s="32"/>
-      <c r="L45" s="32"/>
-      <c r="M45" s="32"/>
-      <c r="N45" s="32"/>
-      <c r="O45" s="32"/>
-      <c r="P45" s="32"/>
-      <c r="Q45" s="32"/>
-      <c r="R45" s="32"/>
-      <c r="S45" s="32"/>
-      <c r="T45" s="32"/>
-      <c r="U45" s="32"/>
-      <c r="V45" s="32"/>
-      <c r="W45" s="32"/>
-      <c r="X45" s="32"/>
-      <c r="Y45" s="32"/>
-      <c r="Z45" s="32"/>
-      <c r="AA45" s="32"/>
-      <c r="AB45" s="32"/>
+      <c r="I45" s="33"/>
+      <c r="J45" s="33"/>
+      <c r="K45" s="33"/>
+      <c r="L45" s="33"/>
+      <c r="M45" s="33"/>
+      <c r="N45" s="33"/>
+      <c r="O45" s="33"/>
+      <c r="P45" s="33"/>
+      <c r="Q45" s="33"/>
+      <c r="R45" s="33"/>
+      <c r="S45" s="33"/>
+      <c r="T45" s="33"/>
+      <c r="U45" s="33"/>
+      <c r="V45" s="33"/>
+      <c r="W45" s="33"/>
+      <c r="X45" s="33"/>
+      <c r="Y45" s="33"/>
+      <c r="Z45" s="33"/>
+      <c r="AA45" s="33"/>
+      <c r="AB45" s="33"/>
     </row>
     <row r="46" ht="15.0" customHeight="1">
-      <c r="A46" s="27" t="s">
+      <c r="A46" s="28" t="s">
         <v>438</v>
       </c>
-      <c r="B46" s="28"/>
-      <c r="C46" s="28"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="28"/>
-      <c r="F46" s="28"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="28"/>
-      <c r="I46" s="28"/>
-      <c r="J46" s="28"/>
-      <c r="K46" s="28"/>
-      <c r="L46" s="28"/>
-      <c r="M46" s="28"/>
-      <c r="N46" s="28"/>
-      <c r="O46" s="28"/>
-      <c r="P46" s="28"/>
-      <c r="Q46" s="28"/>
-      <c r="R46" s="28"/>
-      <c r="S46" s="28"/>
-      <c r="T46" s="28"/>
-      <c r="U46" s="28"/>
-      <c r="V46" s="28"/>
-      <c r="W46" s="28"/>
-      <c r="X46" s="28"/>
-      <c r="Y46" s="28"/>
-      <c r="Z46" s="28"/>
-      <c r="AA46" s="28"/>
-      <c r="AB46" s="28"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="29"/>
+      <c r="F46" s="29"/>
+      <c r="G46" s="29"/>
+      <c r="H46" s="29"/>
+      <c r="I46" s="29"/>
+      <c r="J46" s="29"/>
+      <c r="K46" s="29"/>
+      <c r="L46" s="29"/>
+      <c r="M46" s="29"/>
+      <c r="N46" s="29"/>
+      <c r="O46" s="29"/>
+      <c r="P46" s="29"/>
+      <c r="Q46" s="29"/>
+      <c r="R46" s="29"/>
+      <c r="S46" s="29"/>
+      <c r="T46" s="29"/>
+      <c r="U46" s="29"/>
+      <c r="V46" s="29"/>
+      <c r="W46" s="29"/>
+      <c r="X46" s="29"/>
+      <c r="Y46" s="29"/>
+      <c r="Z46" s="29"/>
+      <c r="AA46" s="29"/>
+      <c r="AB46" s="29"/>
     </row>
     <row r="47" ht="15.0" customHeight="1">
-      <c r="A47" s="29" t="s">
+      <c r="A47" s="30" t="s">
         <v>439</v>
       </c>
-      <c r="B47" s="32"/>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="31">
+      <c r="B47" s="33"/>
+      <c r="C47" s="33"/>
+      <c r="D47" s="33"/>
+      <c r="E47" s="33"/>
+      <c r="F47" s="33"/>
+      <c r="G47" s="33"/>
+      <c r="H47" s="32">
         <v>24.49</v>
       </c>
-      <c r="I47" s="32"/>
-      <c r="J47" s="32"/>
-      <c r="K47" s="32"/>
-      <c r="L47" s="32"/>
-      <c r="M47" s="32"/>
-      <c r="N47" s="32"/>
-      <c r="O47" s="32"/>
-      <c r="P47" s="32"/>
-      <c r="Q47" s="32"/>
-      <c r="R47" s="32"/>
-      <c r="S47" s="32"/>
-      <c r="T47" s="32"/>
-      <c r="U47" s="32"/>
-      <c r="V47" s="32"/>
-      <c r="W47" s="32"/>
-      <c r="X47" s="32"/>
-      <c r="Y47" s="32"/>
-      <c r="Z47" s="32"/>
-      <c r="AA47" s="32"/>
-      <c r="AB47" s="32"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
+      <c r="K47" s="33"/>
+      <c r="L47" s="33"/>
+      <c r="M47" s="33"/>
+      <c r="N47" s="33"/>
+      <c r="O47" s="33"/>
+      <c r="P47" s="33"/>
+      <c r="Q47" s="33"/>
+      <c r="R47" s="33"/>
+      <c r="S47" s="33"/>
+      <c r="T47" s="33"/>
+      <c r="U47" s="33"/>
+      <c r="V47" s="33"/>
+      <c r="W47" s="33"/>
+      <c r="X47" s="33"/>
+      <c r="Y47" s="33"/>
+      <c r="Z47" s="33"/>
+      <c r="AA47" s="33"/>
+      <c r="AB47" s="33"/>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="27" t="s">
+      <c r="A48" s="28" t="s">
         <v>440</v>
       </c>
-      <c r="B48" s="28"/>
-      <c r="C48" s="28"/>
-      <c r="D48" s="28"/>
-      <c r="E48" s="28"/>
-      <c r="F48" s="28"/>
-      <c r="G48" s="28"/>
-      <c r="H48" s="28"/>
-      <c r="I48" s="28"/>
-      <c r="J48" s="28"/>
-      <c r="K48" s="28"/>
-      <c r="L48" s="28"/>
-      <c r="M48" s="28"/>
-      <c r="N48" s="28"/>
-      <c r="O48" s="28"/>
-      <c r="P48" s="28"/>
-      <c r="Q48" s="28"/>
-      <c r="R48" s="28"/>
-      <c r="S48" s="28"/>
-      <c r="T48" s="28"/>
-      <c r="U48" s="28"/>
-      <c r="V48" s="28"/>
-      <c r="W48" s="28"/>
-      <c r="X48" s="28"/>
-      <c r="Y48" s="28"/>
-      <c r="Z48" s="28"/>
-      <c r="AA48" s="28"/>
-      <c r="AB48" s="28"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="29"/>
+      <c r="F48" s="29"/>
+      <c r="G48" s="29"/>
+      <c r="H48" s="29"/>
+      <c r="I48" s="29"/>
+      <c r="J48" s="29"/>
+      <c r="K48" s="29"/>
+      <c r="L48" s="29"/>
+      <c r="M48" s="29"/>
+      <c r="N48" s="29"/>
+      <c r="O48" s="29"/>
+      <c r="P48" s="29"/>
+      <c r="Q48" s="29"/>
+      <c r="R48" s="29"/>
+      <c r="S48" s="29"/>
+      <c r="T48" s="29"/>
+      <c r="U48" s="29"/>
+      <c r="V48" s="29"/>
+      <c r="W48" s="29"/>
+      <c r="X48" s="29"/>
+      <c r="Y48" s="29"/>
+      <c r="Z48" s="29"/>
+      <c r="AA48" s="29"/>
+      <c r="AB48" s="29"/>
     </row>
     <row r="49" ht="15.0" customHeight="1">
-      <c r="A49" s="29" t="s">
+      <c r="A49" s="30" t="s">
         <v>441</v>
       </c>
-      <c r="B49" s="32"/>
-      <c r="C49" s="32"/>
-      <c r="D49" s="32"/>
-      <c r="E49" s="32"/>
-      <c r="F49" s="32"/>
-      <c r="G49" s="31">
+      <c r="B49" s="33"/>
+      <c r="C49" s="33"/>
+      <c r="D49" s="33"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="32">
         <v>95.17</v>
       </c>
-      <c r="H49" s="31">
+      <c r="H49" s="32">
         <v>24.49</v>
       </c>
-      <c r="I49" s="32"/>
-      <c r="J49" s="32"/>
-      <c r="K49" s="32"/>
-      <c r="L49" s="32"/>
-      <c r="M49" s="32"/>
-      <c r="N49" s="32"/>
-      <c r="O49" s="32"/>
-      <c r="P49" s="32"/>
-      <c r="Q49" s="32"/>
-      <c r="R49" s="32"/>
-      <c r="S49" s="32"/>
-      <c r="T49" s="32"/>
-      <c r="U49" s="32"/>
-      <c r="V49" s="32"/>
-      <c r="W49" s="32"/>
-      <c r="X49" s="32"/>
-      <c r="Y49" s="32"/>
-      <c r="Z49" s="32"/>
-      <c r="AA49" s="32"/>
-      <c r="AB49" s="32"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="33"/>
+      <c r="K49" s="33"/>
+      <c r="L49" s="33"/>
+      <c r="M49" s="33"/>
+      <c r="N49" s="33"/>
+      <c r="O49" s="33"/>
+      <c r="P49" s="33"/>
+      <c r="Q49" s="33"/>
+      <c r="R49" s="33"/>
+      <c r="S49" s="33"/>
+      <c r="T49" s="33"/>
+      <c r="U49" s="33"/>
+      <c r="V49" s="33"/>
+      <c r="W49" s="33"/>
+      <c r="X49" s="33"/>
+      <c r="Y49" s="33"/>
+      <c r="Z49" s="33"/>
+      <c r="AA49" s="33"/>
+      <c r="AB49" s="33"/>
     </row>
     <row r="50" ht="15.0" customHeight="1">
-      <c r="A50" s="29" t="s">
+      <c r="A50" s="30" t="s">
         <v>442</v>
       </c>
-      <c r="B50" s="31">
+      <c r="B50" s="32">
         <v>1.1</v>
       </c>
-      <c r="C50" s="31">
+      <c r="C50" s="32">
         <v>1.17</v>
       </c>
-      <c r="D50" s="31">
+      <c r="D50" s="32">
         <v>1.22</v>
       </c>
-      <c r="E50" s="31">
+      <c r="E50" s="32">
         <v>1.27</v>
       </c>
-      <c r="F50" s="31">
+      <c r="F50" s="32">
         <v>1.48</v>
       </c>
-      <c r="G50" s="31">
+      <c r="G50" s="32">
         <v>1.26</v>
       </c>
-      <c r="H50" s="31">
+      <c r="H50" s="32">
         <v>1.69</v>
       </c>
-      <c r="I50" s="31">
+      <c r="I50" s="32">
         <v>2.17</v>
       </c>
-      <c r="J50" s="31">
+      <c r="J50" s="32">
         <v>2.1</v>
       </c>
-      <c r="K50" s="31">
+      <c r="K50" s="32">
         <v>1.63</v>
       </c>
-      <c r="L50" s="31">
+      <c r="L50" s="32">
         <v>1.38</v>
       </c>
-      <c r="M50" s="31">
+      <c r="M50" s="32">
         <v>1.07</v>
       </c>
-      <c r="N50" s="31">
+      <c r="N50" s="32">
         <v>0.7</v>
       </c>
-      <c r="O50" s="31">
+      <c r="O50" s="32">
         <v>1.13</v>
       </c>
-      <c r="P50" s="31">
+      <c r="P50" s="32">
         <v>1.53</v>
       </c>
-      <c r="Q50" s="31">
+      <c r="Q50" s="32">
         <v>2.01</v>
       </c>
-      <c r="R50" s="31">
+      <c r="R50" s="32">
         <v>2.3</v>
       </c>
-      <c r="S50" s="31">
+      <c r="S50" s="32">
         <v>2.86</v>
       </c>
-      <c r="T50" s="31">
+      <c r="T50" s="32">
         <v>3.02</v>
       </c>
-      <c r="U50" s="31">
+      <c r="U50" s="32">
         <v>2.6</v>
       </c>
-      <c r="V50" s="32"/>
-      <c r="W50" s="32"/>
-      <c r="X50" s="32"/>
-      <c r="Y50" s="32"/>
-      <c r="Z50" s="32"/>
-      <c r="AA50" s="32"/>
-      <c r="AB50" s="32"/>
+      <c r="V50" s="33"/>
+      <c r="W50" s="33"/>
+      <c r="X50" s="33"/>
+      <c r="Y50" s="33"/>
+      <c r="Z50" s="33"/>
+      <c r="AA50" s="33"/>
+      <c r="AB50" s="33"/>
     </row>
     <row r="51" ht="15.0" customHeight="1">
-      <c r="A51" s="27" t="s">
+      <c r="A51" s="28" t="s">
         <v>443</v>
       </c>
-      <c r="B51" s="28"/>
-      <c r="C51" s="28"/>
-      <c r="D51" s="28"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="28"/>
-      <c r="G51" s="28"/>
-      <c r="H51" s="28"/>
-      <c r="I51" s="28"/>
-      <c r="J51" s="28"/>
-      <c r="K51" s="28"/>
-      <c r="L51" s="28"/>
-      <c r="M51" s="28"/>
-      <c r="N51" s="28"/>
-      <c r="O51" s="28"/>
-      <c r="P51" s="28"/>
-      <c r="Q51" s="28"/>
-      <c r="R51" s="28"/>
-      <c r="S51" s="28"/>
-      <c r="T51" s="28"/>
-      <c r="U51" s="28"/>
-      <c r="V51" s="28"/>
-      <c r="W51" s="28"/>
-      <c r="X51" s="28"/>
-      <c r="Y51" s="28"/>
-      <c r="Z51" s="28"/>
-      <c r="AA51" s="28"/>
-      <c r="AB51" s="28"/>
+      <c r="B51" s="29"/>
+      <c r="C51" s="29"/>
+      <c r="D51" s="29"/>
+      <c r="E51" s="29"/>
+      <c r="F51" s="29"/>
+      <c r="G51" s="29"/>
+      <c r="H51" s="29"/>
+      <c r="I51" s="29"/>
+      <c r="J51" s="29"/>
+      <c r="K51" s="29"/>
+      <c r="L51" s="29"/>
+      <c r="M51" s="29"/>
+      <c r="N51" s="29"/>
+      <c r="O51" s="29"/>
+      <c r="P51" s="29"/>
+      <c r="Q51" s="29"/>
+      <c r="R51" s="29"/>
+      <c r="S51" s="29"/>
+      <c r="T51" s="29"/>
+      <c r="U51" s="29"/>
+      <c r="V51" s="29"/>
+      <c r="W51" s="29"/>
+      <c r="X51" s="29"/>
+      <c r="Y51" s="29"/>
+      <c r="Z51" s="29"/>
+      <c r="AA51" s="29"/>
+      <c r="AB51" s="29"/>
     </row>
     <row r="52" ht="15.0" customHeight="1">
-      <c r="A52" s="29" t="s">
+      <c r="A52" s="30" t="s">
         <v>444</v>
       </c>
-      <c r="B52" s="32"/>
-      <c r="C52" s="32"/>
-      <c r="D52" s="32"/>
-      <c r="E52" s="32"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="31">
+      <c r="B52" s="33"/>
+      <c r="C52" s="33"/>
+      <c r="D52" s="33"/>
+      <c r="E52" s="33"/>
+      <c r="F52" s="33"/>
+      <c r="G52" s="33"/>
+      <c r="H52" s="32">
         <v>0.18</v>
       </c>
-      <c r="I52" s="32"/>
-      <c r="J52" s="32"/>
-      <c r="K52" s="32"/>
-      <c r="L52" s="32"/>
-      <c r="M52" s="32"/>
-      <c r="N52" s="32"/>
-      <c r="O52" s="32"/>
-      <c r="P52" s="32"/>
-      <c r="Q52" s="32"/>
-      <c r="R52" s="32"/>
-      <c r="S52" s="32"/>
-      <c r="T52" s="32"/>
-      <c r="U52" s="32"/>
-      <c r="V52" s="32"/>
-      <c r="W52" s="32"/>
-      <c r="X52" s="32"/>
-      <c r="Y52" s="32"/>
-      <c r="Z52" s="32"/>
-      <c r="AA52" s="32"/>
-      <c r="AB52" s="32"/>
+      <c r="I52" s="33"/>
+      <c r="J52" s="33"/>
+      <c r="K52" s="33"/>
+      <c r="L52" s="33"/>
+      <c r="M52" s="33"/>
+      <c r="N52" s="33"/>
+      <c r="O52" s="33"/>
+      <c r="P52" s="33"/>
+      <c r="Q52" s="33"/>
+      <c r="R52" s="33"/>
+      <c r="S52" s="33"/>
+      <c r="T52" s="33"/>
+      <c r="U52" s="33"/>
+      <c r="V52" s="33"/>
+      <c r="W52" s="33"/>
+      <c r="X52" s="33"/>
+      <c r="Y52" s="33"/>
+      <c r="Z52" s="33"/>
+      <c r="AA52" s="33"/>
+      <c r="AB52" s="33"/>
     </row>
     <row r="53" ht="15.0" customHeight="1">
-      <c r="A53" s="27" t="s">
+      <c r="A53" s="28" t="s">
         <v>445</v>
       </c>
-      <c r="B53" s="28"/>
-      <c r="C53" s="28"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="28"/>
-      <c r="F53" s="28"/>
-      <c r="G53" s="28"/>
-      <c r="H53" s="28"/>
-      <c r="I53" s="28"/>
-      <c r="J53" s="28"/>
-      <c r="K53" s="28"/>
-      <c r="L53" s="28"/>
-      <c r="M53" s="28"/>
-      <c r="N53" s="28"/>
-      <c r="O53" s="28"/>
-      <c r="P53" s="28"/>
-      <c r="Q53" s="28"/>
-      <c r="R53" s="28"/>
-      <c r="S53" s="28"/>
-      <c r="T53" s="28"/>
-      <c r="U53" s="28"/>
-      <c r="V53" s="28"/>
-      <c r="W53" s="28"/>
-      <c r="X53" s="28"/>
-      <c r="Y53" s="28"/>
-      <c r="Z53" s="28"/>
-      <c r="AA53" s="28"/>
-      <c r="AB53" s="28"/>
+      <c r="B53" s="29"/>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="29"/>
+      <c r="F53" s="29"/>
+      <c r="G53" s="29"/>
+      <c r="H53" s="29"/>
+      <c r="I53" s="29"/>
+      <c r="J53" s="29"/>
+      <c r="K53" s="29"/>
+      <c r="L53" s="29"/>
+      <c r="M53" s="29"/>
+      <c r="N53" s="29"/>
+      <c r="O53" s="29"/>
+      <c r="P53" s="29"/>
+      <c r="Q53" s="29"/>
+      <c r="R53" s="29"/>
+      <c r="S53" s="29"/>
+      <c r="T53" s="29"/>
+      <c r="U53" s="29"/>
+      <c r="V53" s="29"/>
+      <c r="W53" s="29"/>
+      <c r="X53" s="29"/>
+      <c r="Y53" s="29"/>
+      <c r="Z53" s="29"/>
+      <c r="AA53" s="29"/>
+      <c r="AB53" s="29"/>
     </row>
     <row r="54" ht="15.0" customHeight="1">
-      <c r="A54" s="29" t="s">
+      <c r="A54" s="30" t="s">
         <v>446</v>
       </c>
-      <c r="B54" s="31">
+      <c r="B54" s="32">
         <v>0.57</v>
       </c>
-      <c r="C54" s="31">
+      <c r="C54" s="32">
         <v>0.38</v>
       </c>
-      <c r="D54" s="31">
+      <c r="D54" s="32">
         <v>0.38</v>
       </c>
-      <c r="E54" s="31">
+      <c r="E54" s="32">
         <v>0.68</v>
       </c>
-      <c r="F54" s="31">
+      <c r="F54" s="32">
         <v>0.97</v>
       </c>
-      <c r="G54" s="31">
+      <c r="G54" s="32">
         <v>0.49</v>
       </c>
-      <c r="H54" s="31">
+      <c r="H54" s="32">
         <v>0.51</v>
       </c>
-      <c r="I54" s="31">
+      <c r="I54" s="32">
         <v>0.69</v>
       </c>
-      <c r="J54" s="31">
+      <c r="J54" s="32">
         <v>1.23</v>
       </c>
-      <c r="K54" s="31">
+      <c r="K54" s="32">
         <v>0.46</v>
       </c>
-      <c r="L54" s="31">
+      <c r="L54" s="32">
         <v>2.92</v>
       </c>
-      <c r="M54" s="31">
+      <c r="M54" s="32">
         <v>3.66</v>
       </c>
-      <c r="N54" s="31">
+      <c r="N54" s="32">
         <v>1.39</v>
       </c>
-      <c r="O54" s="31">
+      <c r="O54" s="32">
         <v>0.48</v>
       </c>
-      <c r="P54" s="31">
+      <c r="P54" s="32">
         <v>1.05</v>
       </c>
-      <c r="Q54" s="31">
+      <c r="Q54" s="32">
         <v>1.5</v>
       </c>
-      <c r="R54" s="31">
+      <c r="R54" s="32">
         <v>0.88</v>
       </c>
-      <c r="S54" s="31">
+      <c r="S54" s="32">
         <v>6.85</v>
       </c>
-      <c r="T54" s="31">
+      <c r="T54" s="32">
         <v>8.59</v>
       </c>
-      <c r="U54" s="31">
+      <c r="U54" s="32">
         <v>12.66</v>
       </c>
-      <c r="V54" s="31">
+      <c r="V54" s="32">
         <v>4.8</v>
       </c>
-      <c r="W54" s="31">
+      <c r="W54" s="32">
         <v>9.17</v>
       </c>
-      <c r="X54" s="31">
+      <c r="X54" s="32">
         <v>2.02</v>
       </c>
-      <c r="Y54" s="31">
+      <c r="Y54" s="32">
         <v>27.47</v>
       </c>
-      <c r="Z54" s="32"/>
-      <c r="AA54" s="32"/>
-      <c r="AB54" s="32"/>
+      <c r="Z54" s="33"/>
+      <c r="AA54" s="33"/>
+      <c r="AB54" s="33"/>
     </row>
     <row r="55" ht="15.0" customHeight="1">
-      <c r="A55" s="29" t="s">
+      <c r="A55" s="30" t="s">
         <v>447</v>
       </c>
-      <c r="B55" s="31">
+      <c r="B55" s="32">
         <v>0.59</v>
       </c>
-      <c r="C55" s="31">
+      <c r="C55" s="32">
         <v>0.58</v>
       </c>
-      <c r="D55" s="31">
+      <c r="D55" s="32">
         <v>0.6</v>
       </c>
-      <c r="E55" s="31">
+      <c r="E55" s="32">
         <v>0.67</v>
       </c>
-      <c r="F55" s="31">
+      <c r="F55" s="32">
         <v>0.74</v>
       </c>
-      <c r="G55" s="31">
+      <c r="G55" s="32">
         <v>0.63</v>
       </c>
-      <c r="H55" s="31">
+      <c r="H55" s="32">
         <v>0.72</v>
       </c>
-      <c r="I55" s="31">
+      <c r="I55" s="32">
         <v>0.9</v>
       </c>
-      <c r="J55" s="31">
+      <c r="J55" s="32">
         <v>1.03</v>
       </c>
-      <c r="K55" s="31">
+      <c r="K55" s="32">
         <v>0.86</v>
       </c>
-      <c r="L55" s="31">
+      <c r="L55" s="32">
         <v>1.91</v>
       </c>
-      <c r="M55" s="31">
+      <c r="M55" s="32">
         <v>1.61</v>
       </c>
-      <c r="N55" s="31">
+      <c r="N55" s="32">
         <v>1.04</v>
       </c>
-      <c r="O55" s="31">
+      <c r="O55" s="32">
         <v>2.47</v>
       </c>
-      <c r="P55" s="31">
+      <c r="P55" s="32">
         <v>3.59</v>
       </c>
-      <c r="Q55" s="31">
+      <c r="Q55" s="32">
         <v>5.07</v>
       </c>
-      <c r="R55" s="31">
+      <c r="R55" s="32">
         <v>5.7</v>
       </c>
-      <c r="S55" s="31">
+      <c r="S55" s="32">
         <v>7.92</v>
       </c>
-      <c r="T55" s="31">
+      <c r="T55" s="32">
         <v>7.56</v>
       </c>
-      <c r="U55" s="31">
+      <c r="U55" s="32">
         <v>7.76</v>
       </c>
-      <c r="V55" s="32"/>
-      <c r="W55" s="32"/>
-      <c r="X55" s="32"/>
-      <c r="Y55" s="32"/>
-      <c r="Z55" s="32"/>
-      <c r="AA55" s="32"/>
-      <c r="AB55" s="32"/>
+      <c r="V55" s="33"/>
+      <c r="W55" s="33"/>
+      <c r="X55" s="33"/>
+      <c r="Y55" s="33"/>
+      <c r="Z55" s="33"/>
+      <c r="AA55" s="33"/>
+      <c r="AB55" s="33"/>
     </row>
     <row r="56" ht="15.0" customHeight="1">
-      <c r="A56" s="27" t="s">
+      <c r="A56" s="28" t="s">
         <v>448</v>
       </c>
-      <c r="B56" s="28"/>
-      <c r="C56" s="28"/>
-      <c r="D56" s="28"/>
-      <c r="E56" s="28"/>
-      <c r="F56" s="28"/>
-      <c r="G56" s="28"/>
-      <c r="H56" s="28"/>
-      <c r="I56" s="28"/>
-      <c r="J56" s="28"/>
-      <c r="K56" s="28"/>
-      <c r="L56" s="28"/>
-      <c r="M56" s="28"/>
-      <c r="N56" s="28"/>
-      <c r="O56" s="28"/>
-      <c r="P56" s="28"/>
-      <c r="Q56" s="28"/>
-      <c r="R56" s="28"/>
-      <c r="S56" s="28"/>
-      <c r="T56" s="28"/>
-      <c r="U56" s="28"/>
-      <c r="V56" s="28"/>
-      <c r="W56" s="28"/>
-      <c r="X56" s="28"/>
-      <c r="Y56" s="28"/>
-      <c r="Z56" s="28"/>
-      <c r="AA56" s="28"/>
-      <c r="AB56" s="28"/>
+      <c r="B56" s="29"/>
+      <c r="C56" s="29"/>
+      <c r="D56" s="29"/>
+      <c r="E56" s="29"/>
+      <c r="F56" s="29"/>
+      <c r="G56" s="29"/>
+      <c r="H56" s="29"/>
+      <c r="I56" s="29"/>
+      <c r="J56" s="29"/>
+      <c r="K56" s="29"/>
+      <c r="L56" s="29"/>
+      <c r="M56" s="29"/>
+      <c r="N56" s="29"/>
+      <c r="O56" s="29"/>
+      <c r="P56" s="29"/>
+      <c r="Q56" s="29"/>
+      <c r="R56" s="29"/>
+      <c r="S56" s="29"/>
+      <c r="T56" s="29"/>
+      <c r="U56" s="29"/>
+      <c r="V56" s="29"/>
+      <c r="W56" s="29"/>
+      <c r="X56" s="29"/>
+      <c r="Y56" s="29"/>
+      <c r="Z56" s="29"/>
+      <c r="AA56" s="29"/>
+      <c r="AB56" s="29"/>
     </row>
     <row r="57" ht="15.0" customHeight="1">
-      <c r="A57" s="29" t="s">
+      <c r="A57" s="30" t="s">
         <v>449</v>
       </c>
-      <c r="B57" s="31">
+      <c r="B57" s="32">
         <v>4.09</v>
       </c>
-      <c r="C57" s="31">
+      <c r="C57" s="32">
         <v>3.03</v>
       </c>
-      <c r="D57" s="31">
+      <c r="D57" s="32">
         <v>6.27</v>
       </c>
-      <c r="E57" s="31">
+      <c r="E57" s="32">
         <v>16.94</v>
       </c>
-      <c r="F57" s="31">
+      <c r="F57" s="32">
         <v>10.64</v>
       </c>
-      <c r="G57" s="31">
+      <c r="G57" s="32">
         <v>21.31</v>
       </c>
-      <c r="H57" s="31">
+      <c r="H57" s="32">
         <v>12.69</v>
       </c>
-      <c r="I57" s="32"/>
-      <c r="J57" s="32"/>
-      <c r="K57" s="31">
+      <c r="I57" s="33"/>
+      <c r="J57" s="33"/>
+      <c r="K57" s="32">
         <v>11.85</v>
       </c>
-      <c r="L57" s="32"/>
-      <c r="M57" s="32"/>
-      <c r="N57" s="32"/>
-      <c r="O57" s="32"/>
-      <c r="P57" s="32"/>
-      <c r="Q57" s="32"/>
-      <c r="R57" s="31">
+      <c r="L57" s="33"/>
+      <c r="M57" s="33"/>
+      <c r="N57" s="33"/>
+      <c r="O57" s="33"/>
+      <c r="P57" s="33"/>
+      <c r="Q57" s="33"/>
+      <c r="R57" s="32">
         <v>0.54</v>
       </c>
-      <c r="S57" s="32"/>
-      <c r="T57" s="32"/>
-      <c r="U57" s="32"/>
-      <c r="V57" s="32"/>
-      <c r="W57" s="32"/>
-      <c r="X57" s="32"/>
-      <c r="Y57" s="32"/>
-      <c r="Z57" s="32"/>
-      <c r="AA57" s="32"/>
-      <c r="AB57" s="32"/>
+      <c r="S57" s="33"/>
+      <c r="T57" s="33"/>
+      <c r="U57" s="33"/>
+      <c r="V57" s="33"/>
+      <c r="W57" s="33"/>
+      <c r="X57" s="33"/>
+      <c r="Y57" s="33"/>
+      <c r="Z57" s="33"/>
+      <c r="AA57" s="33"/>
+      <c r="AB57" s="33"/>
     </row>
     <row r="58" ht="15.0" customHeight="1">
-      <c r="A58" s="29" t="s">
+      <c r="A58" s="30" t="s">
         <v>450</v>
       </c>
-      <c r="B58" s="31">
+      <c r="B58" s="32">
         <v>6.76</v>
       </c>
-      <c r="C58" s="31">
+      <c r="C58" s="32">
         <v>8.71</v>
       </c>
-      <c r="D58" s="31">
+      <c r="D58" s="32">
         <v>11.83</v>
       </c>
-      <c r="E58" s="31">
+      <c r="E58" s="32">
         <v>16.21</v>
       </c>
-      <c r="F58" s="31">
+      <c r="F58" s="32">
         <v>20.6</v>
       </c>
-      <c r="G58" s="31">
+      <c r="G58" s="32">
         <v>30.0</v>
       </c>
-      <c r="H58" s="31">
+      <c r="H58" s="32">
         <v>43.85</v>
       </c>
-      <c r="I58" s="30">
+      <c r="I58" s="31">
         <v>314.87</v>
       </c>
-      <c r="J58" s="32"/>
-      <c r="K58" s="32"/>
-      <c r="L58" s="32"/>
-      <c r="M58" s="32"/>
-      <c r="N58" s="31">
+      <c r="J58" s="33"/>
+      <c r="K58" s="33"/>
+      <c r="L58" s="33"/>
+      <c r="M58" s="33"/>
+      <c r="N58" s="32">
         <v>5.99</v>
       </c>
-      <c r="O58" s="31">
+      <c r="O58" s="32">
         <v>18.45</v>
       </c>
-      <c r="P58" s="31">
+      <c r="P58" s="32">
         <v>24.5</v>
       </c>
-      <c r="Q58" s="31">
+      <c r="Q58" s="32">
         <v>35.91</v>
       </c>
-      <c r="R58" s="31">
+      <c r="R58" s="32">
         <v>35.38</v>
       </c>
-      <c r="S58" s="32"/>
-      <c r="T58" s="32"/>
-      <c r="U58" s="32"/>
-      <c r="V58" s="32"/>
-      <c r="W58" s="32"/>
-      <c r="X58" s="32"/>
-      <c r="Y58" s="32"/>
-      <c r="Z58" s="32"/>
-      <c r="AA58" s="32"/>
-      <c r="AB58" s="32"/>
+      <c r="S58" s="33"/>
+      <c r="T58" s="33"/>
+      <c r="U58" s="33"/>
+      <c r="V58" s="33"/>
+      <c r="W58" s="33"/>
+      <c r="X58" s="33"/>
+      <c r="Y58" s="33"/>
+      <c r="Z58" s="33"/>
+      <c r="AA58" s="33"/>
+      <c r="AB58" s="33"/>
     </row>
     <row r="59" ht="15.0" customHeight="1">
-      <c r="A59" s="27" t="s">
+      <c r="A59" s="28" t="s">
         <v>451</v>
       </c>
-      <c r="B59" s="28"/>
-      <c r="C59" s="28"/>
-      <c r="D59" s="28"/>
-      <c r="E59" s="28"/>
-      <c r="F59" s="28"/>
-      <c r="G59" s="28"/>
-      <c r="H59" s="28"/>
-      <c r="I59" s="28"/>
-      <c r="J59" s="28"/>
-      <c r="K59" s="28"/>
-      <c r="L59" s="28"/>
-      <c r="M59" s="28"/>
-      <c r="N59" s="28"/>
-      <c r="O59" s="28"/>
-      <c r="P59" s="28"/>
-      <c r="Q59" s="28"/>
-      <c r="R59" s="28"/>
-      <c r="S59" s="28"/>
-      <c r="T59" s="28"/>
-      <c r="U59" s="28"/>
-      <c r="V59" s="28"/>
-      <c r="W59" s="28"/>
-      <c r="X59" s="28"/>
-      <c r="Y59" s="28"/>
-      <c r="Z59" s="28"/>
-      <c r="AA59" s="28"/>
-      <c r="AB59" s="28"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="29"/>
+      <c r="E59" s="29"/>
+      <c r="F59" s="29"/>
+      <c r="G59" s="29"/>
+      <c r="H59" s="29"/>
+      <c r="I59" s="29"/>
+      <c r="J59" s="29"/>
+      <c r="K59" s="29"/>
+      <c r="L59" s="29"/>
+      <c r="M59" s="29"/>
+      <c r="N59" s="29"/>
+      <c r="O59" s="29"/>
+      <c r="P59" s="29"/>
+      <c r="Q59" s="29"/>
+      <c r="R59" s="29"/>
+      <c r="S59" s="29"/>
+      <c r="T59" s="29"/>
+      <c r="U59" s="29"/>
+      <c r="V59" s="29"/>
+      <c r="W59" s="29"/>
+      <c r="X59" s="29"/>
+      <c r="Y59" s="29"/>
+      <c r="Z59" s="29"/>
+      <c r="AA59" s="29"/>
+      <c r="AB59" s="29"/>
     </row>
     <row r="60" ht="15.0" customHeight="1">
-      <c r="A60" s="29" t="s">
+      <c r="A60" s="30" t="s">
         <v>452</v>
       </c>
-      <c r="B60" s="31">
+      <c r="B60" s="32">
         <v>4.95</v>
       </c>
-      <c r="C60" s="31">
+      <c r="C60" s="32">
         <v>2.91</v>
       </c>
-      <c r="D60" s="31">
+      <c r="D60" s="32">
         <v>3.87</v>
       </c>
-      <c r="E60" s="31">
+      <c r="E60" s="32">
         <v>6.82</v>
       </c>
-      <c r="F60" s="31">
+      <c r="F60" s="32">
         <v>15.63</v>
       </c>
-      <c r="G60" s="31">
+      <c r="G60" s="32">
         <v>10.41</v>
       </c>
-      <c r="H60" s="31">
+      <c r="H60" s="32">
         <v>19.9</v>
       </c>
-      <c r="I60" s="32"/>
-      <c r="J60" s="32"/>
-      <c r="K60" s="31">
+      <c r="I60" s="33"/>
+      <c r="J60" s="33"/>
+      <c r="K60" s="32">
         <v>8.28</v>
       </c>
-      <c r="L60" s="32"/>
-      <c r="M60" s="32"/>
-      <c r="N60" s="32"/>
-      <c r="O60" s="32"/>
-      <c r="P60" s="32"/>
-      <c r="Q60" s="32"/>
-      <c r="R60" s="32"/>
-      <c r="S60" s="32"/>
-      <c r="T60" s="32"/>
-      <c r="U60" s="32"/>
-      <c r="V60" s="32"/>
-      <c r="W60" s="32"/>
-      <c r="X60" s="32"/>
-      <c r="Y60" s="32"/>
-      <c r="Z60" s="32"/>
-      <c r="AA60" s="32"/>
-      <c r="AB60" s="32"/>
+      <c r="L60" s="33"/>
+      <c r="M60" s="33"/>
+      <c r="N60" s="33"/>
+      <c r="O60" s="33"/>
+      <c r="P60" s="33"/>
+      <c r="Q60" s="33"/>
+      <c r="R60" s="33"/>
+      <c r="S60" s="33"/>
+      <c r="T60" s="33"/>
+      <c r="U60" s="33"/>
+      <c r="V60" s="33"/>
+      <c r="W60" s="33"/>
+      <c r="X60" s="33"/>
+      <c r="Y60" s="33"/>
+      <c r="Z60" s="33"/>
+      <c r="AA60" s="33"/>
+      <c r="AB60" s="33"/>
     </row>
     <row r="61" ht="15.0" customHeight="1">
-      <c r="A61" s="29" t="s">
+      <c r="A61" s="30" t="s">
         <v>453</v>
       </c>
-      <c r="B61" s="31">
+      <c r="B61" s="32">
         <v>5.93</v>
       </c>
-      <c r="C61" s="31">
+      <c r="C61" s="32">
         <v>6.62</v>
       </c>
-      <c r="D61" s="31">
+      <c r="D61" s="32">
         <v>8.81</v>
       </c>
-      <c r="E61" s="31">
+      <c r="E61" s="32">
         <v>14.74</v>
       </c>
-      <c r="F61" s="31">
+      <c r="F61" s="32">
         <v>40.19</v>
       </c>
-      <c r="G61" s="31">
+      <c r="G61" s="32">
         <v>52.78</v>
       </c>
-      <c r="H61" s="32"/>
-      <c r="I61" s="32"/>
-      <c r="J61" s="32"/>
-      <c r="K61" s="32"/>
-      <c r="L61" s="32"/>
-      <c r="M61" s="32"/>
-      <c r="N61" s="32"/>
-      <c r="O61" s="32"/>
-      <c r="P61" s="32"/>
-      <c r="Q61" s="32"/>
-      <c r="R61" s="32"/>
-      <c r="S61" s="32"/>
-      <c r="T61" s="32"/>
-      <c r="U61" s="32"/>
-      <c r="V61" s="32"/>
-      <c r="W61" s="32"/>
-      <c r="X61" s="32"/>
-      <c r="Y61" s="32"/>
-      <c r="Z61" s="32"/>
-      <c r="AA61" s="32"/>
-      <c r="AB61" s="32"/>
+      <c r="H61" s="33"/>
+      <c r="I61" s="33"/>
+      <c r="J61" s="33"/>
+      <c r="K61" s="33"/>
+      <c r="L61" s="33"/>
+      <c r="M61" s="33"/>
+      <c r="N61" s="33"/>
+      <c r="O61" s="33"/>
+      <c r="P61" s="33"/>
+      <c r="Q61" s="33"/>
+      <c r="R61" s="33"/>
+      <c r="S61" s="33"/>
+      <c r="T61" s="33"/>
+      <c r="U61" s="33"/>
+      <c r="V61" s="33"/>
+      <c r="W61" s="33"/>
+      <c r="X61" s="33"/>
+      <c r="Y61" s="33"/>
+      <c r="Z61" s="33"/>
+      <c r="AA61" s="33"/>
+      <c r="AB61" s="33"/>
     </row>
     <row r="62" ht="15.0" customHeight="1">
-      <c r="A62" s="27" t="s">
+      <c r="A62" s="28" t="s">
         <v>454</v>
       </c>
-      <c r="B62" s="28"/>
-      <c r="C62" s="28"/>
-      <c r="D62" s="28"/>
-      <c r="E62" s="28"/>
-      <c r="F62" s="28"/>
-      <c r="G62" s="28"/>
-      <c r="H62" s="28"/>
-      <c r="I62" s="28"/>
-      <c r="J62" s="28"/>
-      <c r="K62" s="28"/>
-      <c r="L62" s="28"/>
-      <c r="M62" s="28"/>
-      <c r="N62" s="28"/>
-      <c r="O62" s="28"/>
-      <c r="P62" s="28"/>
-      <c r="Q62" s="28"/>
-      <c r="R62" s="28"/>
-      <c r="S62" s="28"/>
-      <c r="T62" s="28"/>
-      <c r="U62" s="28"/>
-      <c r="V62" s="28"/>
-      <c r="W62" s="28"/>
-      <c r="X62" s="28"/>
-      <c r="Y62" s="28"/>
-      <c r="Z62" s="28"/>
-      <c r="AA62" s="28"/>
-      <c r="AB62" s="28"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="29"/>
+      <c r="E62" s="29"/>
+      <c r="F62" s="29"/>
+      <c r="G62" s="29"/>
+      <c r="H62" s="29"/>
+      <c r="I62" s="29"/>
+      <c r="J62" s="29"/>
+      <c r="K62" s="29"/>
+      <c r="L62" s="29"/>
+      <c r="M62" s="29"/>
+      <c r="N62" s="29"/>
+      <c r="O62" s="29"/>
+      <c r="P62" s="29"/>
+      <c r="Q62" s="29"/>
+      <c r="R62" s="29"/>
+      <c r="S62" s="29"/>
+      <c r="T62" s="29"/>
+      <c r="U62" s="29"/>
+      <c r="V62" s="29"/>
+      <c r="W62" s="29"/>
+      <c r="X62" s="29"/>
+      <c r="Y62" s="29"/>
+      <c r="Z62" s="29"/>
+      <c r="AA62" s="29"/>
+      <c r="AB62" s="29"/>
     </row>
     <row r="63" ht="15.0" customHeight="1">
-      <c r="A63" s="29" t="s">
+      <c r="A63" s="30" t="s">
         <v>455</v>
       </c>
-      <c r="B63" s="32"/>
-      <c r="C63" s="32"/>
-      <c r="D63" s="32"/>
-      <c r="E63" s="32"/>
-      <c r="F63" s="32"/>
-      <c r="G63" s="31">
+      <c r="B63" s="33"/>
+      <c r="C63" s="33"/>
+      <c r="D63" s="33"/>
+      <c r="E63" s="33"/>
+      <c r="F63" s="33"/>
+      <c r="G63" s="32">
         <v>28.3</v>
       </c>
-      <c r="H63" s="31">
+      <c r="H63" s="32">
         <v>34.76</v>
       </c>
-      <c r="I63" s="32"/>
-      <c r="J63" s="32"/>
-      <c r="K63" s="31">
+      <c r="I63" s="33"/>
+      <c r="J63" s="33"/>
+      <c r="K63" s="32">
         <v>8.46</v>
       </c>
-      <c r="L63" s="32"/>
-      <c r="M63" s="32"/>
-      <c r="N63" s="32"/>
-      <c r="O63" s="32"/>
-      <c r="P63" s="32"/>
-      <c r="Q63" s="32"/>
-      <c r="R63" s="32"/>
-      <c r="S63" s="32"/>
-      <c r="T63" s="32"/>
-      <c r="U63" s="32"/>
-      <c r="V63" s="32"/>
-      <c r="W63" s="32"/>
-      <c r="X63" s="32"/>
-      <c r="Y63" s="32"/>
-      <c r="Z63" s="32"/>
-      <c r="AA63" s="32"/>
-      <c r="AB63" s="32"/>
+      <c r="L63" s="33"/>
+      <c r="M63" s="33"/>
+      <c r="N63" s="33"/>
+      <c r="O63" s="33"/>
+      <c r="P63" s="33"/>
+      <c r="Q63" s="33"/>
+      <c r="R63" s="33"/>
+      <c r="S63" s="33"/>
+      <c r="T63" s="33"/>
+      <c r="U63" s="33"/>
+      <c r="V63" s="33"/>
+      <c r="W63" s="33"/>
+      <c r="X63" s="33"/>
+      <c r="Y63" s="33"/>
+      <c r="Z63" s="33"/>
+      <c r="AA63" s="33"/>
+      <c r="AB63" s="33"/>
     </row>
     <row r="64" ht="15.0" customHeight="1">
-      <c r="A64" s="29" t="s">
+      <c r="A64" s="30" t="s">
         <v>456</v>
       </c>
-      <c r="B64" s="32"/>
-      <c r="C64" s="32"/>
-      <c r="D64" s="32"/>
-      <c r="E64" s="32"/>
-      <c r="F64" s="32"/>
-      <c r="G64" s="30">
+      <c r="B64" s="33"/>
+      <c r="C64" s="33"/>
+      <c r="D64" s="33"/>
+      <c r="E64" s="33"/>
+      <c r="F64" s="33"/>
+      <c r="G64" s="31">
         <v>4268.45</v>
       </c>
-      <c r="H64" s="32"/>
-      <c r="I64" s="32"/>
-      <c r="J64" s="32"/>
-      <c r="K64" s="32"/>
-      <c r="L64" s="32"/>
-      <c r="M64" s="32"/>
-      <c r="N64" s="32"/>
-      <c r="O64" s="32"/>
-      <c r="P64" s="32"/>
-      <c r="Q64" s="32"/>
-      <c r="R64" s="32"/>
-      <c r="S64" s="32"/>
-      <c r="T64" s="32"/>
-      <c r="U64" s="32"/>
-      <c r="V64" s="32"/>
-      <c r="W64" s="32"/>
-      <c r="X64" s="32"/>
-      <c r="Y64" s="32"/>
-      <c r="Z64" s="32"/>
-      <c r="AA64" s="32"/>
-      <c r="AB64" s="32"/>
+      <c r="H64" s="33"/>
+      <c r="I64" s="33"/>
+      <c r="J64" s="33"/>
+      <c r="K64" s="33"/>
+      <c r="L64" s="33"/>
+      <c r="M64" s="33"/>
+      <c r="N64" s="33"/>
+      <c r="O64" s="33"/>
+      <c r="P64" s="33"/>
+      <c r="Q64" s="33"/>
+      <c r="R64" s="33"/>
+      <c r="S64" s="33"/>
+      <c r="T64" s="33"/>
+      <c r="U64" s="33"/>
+      <c r="V64" s="33"/>
+      <c r="W64" s="33"/>
+      <c r="X64" s="33"/>
+      <c r="Y64" s="33"/>
+      <c r="Z64" s="33"/>
+      <c r="AA64" s="33"/>
+      <c r="AB64" s="33"/>
     </row>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>

</xml_diff>